<commit_message>
Align market sizing to Aida's finalized pack-led business plan
The finalized BP flipped from PAYG-led to pack-led, which changes the pricing
engine the bottoms-up sits on:

- PAYG base $15 -> $14.
- Top tier is now the Enterprise 1,000-test pack at $11,200 ($11.20/test, -20%);
  removed the invented flat $30k enterprise fee (not in the BP). All four tiers
  are per-test; ACV = tests/account x blended net price.
- Pack mix shifted pack-led (PAYG 10 / Small 35 / Medium 35 / Enterprise 20)
  vs the old PAYG-heavy 30/30/20/15/5.
- Blended net price $13.58 -> $12.22/test. Retention 85% -> 90% (BP base 93%).

Result: TAM $1.20B -> $0.64B, SAM $144M -> $77M, SOM $2.22M -> $1.34M
(channel ~59% / direct ~41%). SOM now ties to the BP, landing between its
2028 ($1.13M) and 2029 ($2.6M) test-pack revenue. 0 formula error cells.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RsCNYhV2EbucLSqzkWAFLN
</commit_message>
<xml_diff>
--- a/Invirtus_Market_Sizing.xlsx
+++ b/Invirtus_Market_Sizing.xlsx
@@ -672,7 +672,7 @@
     <row r="7">
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Lead with SOM. Reachable 3-year revenue is driven first by the Manatal channel (embedded attach ~56% of SOM), then self-serve. The single biggest assumption is the Year-3 channel attach rate on the ICP-relevant Manatal base (Assumptions sec. 7). Tests/account and the $15 PAYG price are the next two swing factors (see Sensitivity).</t>
+          <t>Lead with SOM. Reachable 3-year revenue is driven first by the Manatal channel (embedded attach ~56% of SOM), then self-serve. The single biggest assumption is the Year-3 channel attach rate on the ICP-relevant Manatal base (Assumptions sec. 7). Tests/account and the $14 PAYG price are the next two swing factors (see Sensitivity).</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -841,7 +841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F91"/>
+  <dimension ref="B1:F89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -1556,7 +1556,7 @@
         </is>
       </c>
       <c r="C36" s="25" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D36" s="21" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
       </c>
       <c r="F36" s="21" t="inlineStr">
         <is>
-          <t>Given. Benchmark: TestGorilla ~$4.3/candidate (Core), TestDome $7-20, HackerRank $15-20, Adaface entry $15. $15 sits at premium end.</t>
+          <t>Finalized BP base (was $15). Benchmark: TestGorilla ~$4.3/candidate, TestDome $7-20, HackerRank $15-20, Adaface entry $15. $14 sits at premium end.</t>
         </is>
       </c>
     </row>
@@ -1619,7 +1619,7 @@
     <row r="39">
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>Large pack discount (200 tests)</t>
+          <t>Enterprise pack discount (1,000 tests)</t>
         </is>
       </c>
       <c r="C39" s="26" t="n">
@@ -1633,7 +1633,7 @@
       <c r="E39" s="22" t="inlineStr"/>
       <c r="F39" s="21" t="inlineStr">
         <is>
-          <t>Given.</t>
+          <t>Finalized BP top tier: 1,000-test Enterprise pack at $11,200 (= $11.20/test). Replaces old 200-unit Large and the flat enterprise fee.</t>
         </is>
       </c>
     </row>
@@ -1694,7 +1694,7 @@
     <row r="43">
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Net price - Large</t>
+          <t xml:space="preserve">   Net price - Enterprise (1,000-pack)</t>
         </is>
       </c>
       <c r="C43" s="27">
@@ -1712,7 +1712,7 @@
     <row r="44" ht="20" customHeight="1">
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>4.  Pack mix  (share of accounts on each plan)</t>
+          <t>4.  Pack mix  (share of accounts on each plan)  [pack-led per finalized BP]</t>
         </is>
       </c>
       <c r="C44" s="5" t="n"/>
@@ -1727,7 +1727,7 @@
         </is>
       </c>
       <c r="C45" s="26" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="D45" s="21" t="inlineStr">
         <is>
@@ -1735,7 +1735,11 @@
         </is>
       </c>
       <c r="E45" s="22" t="inlineStr"/>
-      <c r="F45" s="21" t="inlineStr"/>
+      <c r="F45" s="21" t="inlineStr">
+        <is>
+          <t>Finalized BP is pack-led; PAYG is a thin trial tier, not the base.</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="B46" s="14" t="inlineStr">
@@ -1744,7 +1748,7 @@
         </is>
       </c>
       <c r="C46" s="26" t="n">
-        <v>0.3</v>
+        <v>0.35</v>
       </c>
       <c r="D46" s="21" t="inlineStr">
         <is>
@@ -1761,7 +1765,7 @@
         </is>
       </c>
       <c r="C47" s="26" t="n">
-        <v>0.2</v>
+        <v>0.35</v>
       </c>
       <c r="D47" s="21" t="inlineStr">
         <is>
@@ -1774,11 +1778,11 @@
     <row r="48">
       <c r="B48" s="14" t="inlineStr">
         <is>
-          <t>Large pack share</t>
+          <t>Enterprise (1,000-pack) share</t>
         </is>
       </c>
       <c r="C48" s="26" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="D48" s="21" t="inlineStr">
         <is>
@@ -1786,16 +1790,21 @@
         </is>
       </c>
       <c r="E48" s="22" t="inlineStr"/>
-      <c r="F48" s="21" t="inlineStr"/>
+      <c r="F48" s="21" t="inlineStr">
+        <is>
+          <t>Heaviest buyers; matches finalized BP customer mix.</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="B49" s="14" t="inlineStr">
         <is>
-          <t>Enterprise (unlimited) share</t>
-        </is>
-      </c>
-      <c r="C49" s="26" t="n">
-        <v>0.05</v>
+          <t xml:space="preserve">   Mix check (=100%)</t>
+        </is>
+      </c>
+      <c r="C49" s="28">
+        <f>Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48</f>
+        <v/>
       </c>
       <c r="D49" s="21" t="inlineStr">
         <is>
@@ -1805,366 +1814,363 @@
       <c r="E49" s="22" t="inlineStr"/>
       <c r="F49" s="21" t="inlineStr">
         <is>
-          <t>Larger accounts on a flat custom plan.</t>
+          <t>Must equal 100%.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="B50" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mix check (=100%)</t>
-        </is>
-      </c>
-      <c r="C50" s="28">
-        <f>Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48+Assumptions!$C$49</f>
+          <t xml:space="preserve">   Blended net price per test</t>
+        </is>
+      </c>
+      <c r="C50" s="27">
+        <f>(Assumptions!$C$45*Assumptions!$C$40+Assumptions!$C$46*Assumptions!$C$41+Assumptions!$C$47*Assumptions!$C$42+Assumptions!$C$48*Assumptions!$C$43)/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)</f>
         <v/>
       </c>
       <c r="D50" s="21" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>$/test</t>
         </is>
       </c>
       <c r="E50" s="22" t="inlineStr"/>
       <c r="F50" s="21" t="inlineStr">
         <is>
-          <t>Must equal 100%.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="B51" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Blended net price per test (ex-ent)</t>
-        </is>
-      </c>
-      <c r="C51" s="27">
-        <f>(Assumptions!$C$45*Assumptions!$C$40+Assumptions!$C$46*Assumptions!$C$41+Assumptions!$C$47*Assumptions!$C$42+Assumptions!$C$48*Assumptions!$C$43)/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)</f>
-        <v/>
-      </c>
-      <c r="D51" s="21" t="inlineStr">
-        <is>
-          <t>$/test</t>
-        </is>
-      </c>
-      <c r="E51" s="22" t="inlineStr"/>
-      <c r="F51" s="21" t="inlineStr">
-        <is>
-          <t>Mix-weighted net price of the four per-test packs.</t>
-        </is>
-      </c>
+          <t>Mix-weighted net price across all four packs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>5.  Tests per account / year  (roles x candidates per role)</t>
+        </is>
+      </c>
+      <c r="C51" s="5" t="n"/>
+      <c r="D51" s="5" t="n"/>
+      <c r="E51" s="5" t="n"/>
+      <c r="F51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="B52" s="14" t="inlineStr">
         <is>
-          <t>Enterprise flat annual fee</t>
-        </is>
-      </c>
-      <c r="C52" s="20" t="n">
-        <v>30000</v>
+          <t>Tests-per-account scalar (sensitivity handle)</t>
+        </is>
+      </c>
+      <c r="C52" s="29" t="n">
+        <v>1</v>
       </c>
       <c r="D52" s="21" t="inlineStr">
         <is>
-          <t>$/yr</t>
-        </is>
-      </c>
-      <c r="E52" s="22" t="inlineStr">
-        <is>
-          <t>S7</t>
-        </is>
-      </c>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="E52" s="22" t="inlineStr"/>
       <c r="F52" s="21" t="inlineStr">
         <is>
-          <t>Benchmark: Adaface Enterprise $20k, Unlimited $50k. Implies &lt;$12/test above ~2,500 tests/yr.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="20" customHeight="1">
-      <c r="B53" s="4" t="inlineStr">
-        <is>
-          <t>5.  Tests per account / year  (roles x candidates per role)</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="n"/>
-      <c r="D53" s="5" t="n"/>
-      <c r="E53" s="5" t="n"/>
-      <c r="F53" s="5" t="n"/>
+          <t>Global multiplier on tests/account. Base=1.00; flex in sensitivity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="B53" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Agencies - roles hired / yr</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="n">
+        <v>80</v>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>roles</t>
+        </is>
+      </c>
+      <c r="E53" s="22" t="inlineStr"/>
+      <c r="F53" s="21" t="inlineStr">
+        <is>
+          <t>High req throughput - many client roles, several candidates screened each.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="B54" s="14" t="inlineStr">
         <is>
-          <t>Tests-per-account scalar (sensitivity handle)</t>
-        </is>
-      </c>
-      <c r="C54" s="29" t="n">
-        <v>1</v>
+          <t xml:space="preserve">   Agencies - candidates tested / role</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="n">
+        <v>6</v>
       </c>
       <c r="D54" s="21" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>cand</t>
         </is>
       </c>
       <c r="E54" s="22" t="inlineStr"/>
-      <c r="F54" s="21" t="inlineStr">
-        <is>
-          <t>Global multiplier on tests/account. Base=1.00; flex in sensitivity.</t>
-        </is>
-      </c>
+      <c r="F54" s="21" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="B55" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Agencies - roles hired / yr</t>
-        </is>
-      </c>
-      <c r="C55" s="20" t="n">
-        <v>80</v>
+          <t xml:space="preserve">   Agencies - tests / account / yr</t>
+        </is>
+      </c>
+      <c r="C55" s="23">
+        <f>Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52</f>
+        <v/>
       </c>
       <c r="D55" s="21" t="inlineStr">
         <is>
-          <t>roles</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="E55" s="22" t="inlineStr"/>
       <c r="F55" s="21" t="inlineStr">
         <is>
-          <t>High req throughput - many client roles, several candidates screened each.</t>
+          <t>roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Agencies - candidates tested / role</t>
+          <t xml:space="preserve">   Eng-heavy firms - roles hired / yr</t>
         </is>
       </c>
       <c r="C56" s="20" t="n">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="D56" s="21" t="inlineStr">
         <is>
-          <t>cand</t>
+          <t>roles</t>
         </is>
       </c>
       <c r="E56" s="22" t="inlineStr"/>
-      <c r="F56" s="21" t="inlineStr"/>
+      <c r="F56" s="21" t="inlineStr">
+        <is>
+          <t>Steady in-house eng hiring.</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="B57" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Agencies - tests / account / yr</t>
-        </is>
-      </c>
-      <c r="C57" s="23">
-        <f>Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54</f>
-        <v/>
+          <t xml:space="preserve">   Eng-heavy firms - candidates tested / role</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="n">
+        <v>6</v>
       </c>
       <c r="D57" s="21" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>cand</t>
         </is>
       </c>
       <c r="E57" s="22" t="inlineStr"/>
-      <c r="F57" s="21" t="inlineStr">
-        <is>
-          <t>roles x candidates x scalar.</t>
-        </is>
-      </c>
+      <c r="F57" s="21" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="B58" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Eng-heavy firms - roles hired / yr</t>
-        </is>
-      </c>
-      <c r="C58" s="20" t="n">
-        <v>25</v>
+          <t xml:space="preserve">   Eng-heavy firms - tests / account / yr</t>
+        </is>
+      </c>
+      <c r="C58" s="23">
+        <f>Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52</f>
+        <v/>
       </c>
       <c r="D58" s="21" t="inlineStr">
         <is>
-          <t>roles</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="E58" s="22" t="inlineStr"/>
       <c r="F58" s="21" t="inlineStr">
         <is>
-          <t>Steady in-house eng hiring.</t>
+          <t>roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Eng-heavy firms - candidates tested / role</t>
+          <t xml:space="preserve">   Mid-size firms - roles hired / yr</t>
         </is>
       </c>
       <c r="C59" s="20" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D59" s="21" t="inlineStr">
         <is>
-          <t>cand</t>
+          <t>roles</t>
         </is>
       </c>
       <c r="E59" s="22" t="inlineStr"/>
-      <c r="F59" s="21" t="inlineStr"/>
+      <c r="F59" s="21" t="inlineStr">
+        <is>
+          <t>Sporadic, lower-volume hiring.</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="B60" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Eng-heavy firms - tests / account / yr</t>
-        </is>
-      </c>
-      <c r="C60" s="23">
-        <f>Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54</f>
-        <v/>
+          <t xml:space="preserve">   Mid-size firms - candidates tested / role</t>
+        </is>
+      </c>
+      <c r="C60" s="20" t="n">
+        <v>5</v>
       </c>
       <c r="D60" s="21" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>cand</t>
         </is>
       </c>
       <c r="E60" s="22" t="inlineStr"/>
-      <c r="F60" s="21" t="inlineStr">
-        <is>
-          <t>roles x candidates x scalar.</t>
-        </is>
-      </c>
+      <c r="F60" s="21" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="B61" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mid-size firms - roles hired / yr</t>
-        </is>
-      </c>
-      <c r="C61" s="20" t="n">
-        <v>10</v>
+          <t xml:space="preserve">   Mid-size firms - tests / account / yr</t>
+        </is>
+      </c>
+      <c r="C61" s="23">
+        <f>Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52</f>
+        <v/>
       </c>
       <c r="D61" s="21" t="inlineStr">
         <is>
-          <t>roles</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="E61" s="22" t="inlineStr"/>
       <c r="F61" s="21" t="inlineStr">
         <is>
-          <t>Sporadic, lower-volume hiring.</t>
+          <t>roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="B62" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mid-size firms - candidates tested / role</t>
+          <t xml:space="preserve">   Channel acct - roles hired / yr</t>
         </is>
       </c>
       <c r="C62" s="20" t="n">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="D62" s="21" t="inlineStr">
         <is>
-          <t>cand</t>
+          <t>roles</t>
         </is>
       </c>
       <c r="E62" s="22" t="inlineStr"/>
-      <c r="F62" s="21" t="inlineStr"/>
+      <c r="F62" s="21" t="inlineStr">
+        <is>
+          <t>Manatal users: mix of agencies + in-house recruiters.</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="B63" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Mid-size firms - tests / account / yr</t>
-        </is>
-      </c>
-      <c r="C63" s="23">
-        <f>Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54</f>
-        <v/>
+          <t xml:space="preserve">   Channel acct - candidates tested / role</t>
+        </is>
+      </c>
+      <c r="C63" s="20" t="n">
+        <v>5</v>
       </c>
       <c r="D63" s="21" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>cand</t>
         </is>
       </c>
       <c r="E63" s="22" t="inlineStr"/>
-      <c r="F63" s="21" t="inlineStr">
-        <is>
-          <t>roles x candidates x scalar.</t>
-        </is>
-      </c>
+      <c r="F63" s="21" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="B64" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Channel acct - roles hired / yr</t>
-        </is>
-      </c>
-      <c r="C64" s="20" t="n">
-        <v>40</v>
+          <t xml:space="preserve">   Channel acct - tests / account / yr</t>
+        </is>
+      </c>
+      <c r="C64" s="23">
+        <f>Assumptions!$C$62*Assumptions!$C$63*Assumptions!$C$52</f>
+        <v/>
       </c>
       <c r="D64" s="21" t="inlineStr">
         <is>
-          <t>roles</t>
+          <t>tests</t>
         </is>
       </c>
       <c r="E64" s="22" t="inlineStr"/>
-      <c r="F64" s="21" t="inlineStr">
-        <is>
-          <t>Manatal users: mix of agencies + in-house recruiters.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="B65" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Channel acct - candidates tested / role</t>
-        </is>
-      </c>
-      <c r="C65" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="D65" s="21" t="inlineStr">
-        <is>
-          <t>cand</t>
-        </is>
-      </c>
-      <c r="E65" s="22" t="inlineStr"/>
-      <c r="F65" s="21" t="inlineStr"/>
+      <c r="F64" s="21" t="inlineStr"/>
+    </row>
+    <row r="65" ht="20" customHeight="1">
+      <c r="B65" s="4" t="inlineStr">
+        <is>
+          <t>6.  ACV per account  (revenue/yr)</t>
+        </is>
+      </c>
+      <c r="C65" s="5" t="n"/>
+      <c r="D65" s="5" t="n"/>
+      <c r="E65" s="5" t="n"/>
+      <c r="F65" s="5" t="n"/>
     </row>
     <row r="66">
       <c r="B66" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Channel acct - tests / account / yr</t>
+          <t xml:space="preserve">   Agencies - ACV / account / yr</t>
         </is>
       </c>
       <c r="C66" s="23">
-        <f>Assumptions!$C$64*Assumptions!$C$65*Assumptions!$C$54</f>
+        <f>Assumptions!$C$55*Assumptions!$C$50</f>
         <v/>
       </c>
       <c r="D66" s="21" t="inlineStr">
         <is>
-          <t>tests</t>
+          <t>$/yr</t>
         </is>
       </c>
       <c r="E66" s="22" t="inlineStr"/>
-      <c r="F66" s="21" t="inlineStr"/>
-    </row>
-    <row r="67" ht="20" customHeight="1">
-      <c r="B67" s="4" t="inlineStr">
-        <is>
-          <t>6.  ACV per account  (revenue/yr)</t>
-        </is>
-      </c>
-      <c r="C67" s="5" t="n"/>
-      <c r="D67" s="5" t="n"/>
-      <c r="E67" s="5" t="n"/>
-      <c r="F67" s="5" t="n"/>
+      <c r="F66" s="21" t="inlineStr">
+        <is>
+          <t>tests/account x blended net price per test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="B67" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Eng-heavy firms - ACV / account / yr</t>
+        </is>
+      </c>
+      <c r="C67" s="23">
+        <f>Assumptions!$C$58*Assumptions!$C$50</f>
+        <v/>
+      </c>
+      <c r="D67" s="21" t="inlineStr">
+        <is>
+          <t>$/yr</t>
+        </is>
+      </c>
+      <c r="E67" s="22" t="inlineStr"/>
+      <c r="F67" s="21" t="inlineStr">
+        <is>
+          <t>tests/account x blended net price per test.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="B68" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Agencies - ACV / account / yr</t>
+          <t xml:space="preserve">   Mid-size firms - ACV / account / yr</t>
         </is>
       </c>
       <c r="C68" s="23">
-        <f>(1-Assumptions!$C$49)*(Assumptions!$C$57*Assumptions!$C$51)+Assumptions!$C$49*Assumptions!$C$52</f>
+        <f>Assumptions!$C$61*Assumptions!$C$50</f>
         <v/>
       </c>
       <c r="D68" s="21" t="inlineStr">
@@ -2175,18 +2181,18 @@
       <c r="E68" s="22" t="inlineStr"/>
       <c r="F68" s="21" t="inlineStr">
         <is>
-          <t>(1-ent%) x tests x blended price + ent% x flat fee.</t>
+          <t>tests/account x blended net price per test.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="B69" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Eng-heavy firms - ACV / account / yr</t>
+          <t xml:space="preserve">   Channel acct - ACV / account / yr</t>
         </is>
       </c>
       <c r="C69" s="23">
-        <f>(1-Assumptions!$C$49)*(Assumptions!$C$60*Assumptions!$C$51)+Assumptions!$C$49*Assumptions!$C$52</f>
+        <f>Assumptions!$C$64*Assumptions!$C$50</f>
         <v/>
       </c>
       <c r="D69" s="21" t="inlineStr">
@@ -2197,98 +2203,96 @@
       <c r="E69" s="22" t="inlineStr"/>
       <c r="F69" s="21" t="inlineStr">
         <is>
-          <t>(1-ent%) x tests x blended price + ent% x flat fee.</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="B70" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Mid-size firms - ACV / account / yr</t>
-        </is>
-      </c>
-      <c r="C70" s="23">
-        <f>(1-Assumptions!$C$49)*(Assumptions!$C$63*Assumptions!$C$51)+Assumptions!$C$49*Assumptions!$C$52</f>
-        <v/>
-      </c>
-      <c r="D70" s="21" t="inlineStr">
-        <is>
-          <t>$/yr</t>
-        </is>
-      </c>
-      <c r="E70" s="22" t="inlineStr"/>
-      <c r="F70" s="21" t="inlineStr">
-        <is>
-          <t>(1-ent%) x tests x blended price + ent% x flat fee.</t>
-        </is>
-      </c>
+          <t>tests/account x blended net price per test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="20" customHeight="1">
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>7.  SOM - Channel route (Manatal embedded)  [anchor 10,000+]</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="n"/>
+      <c r="D70" s="5" t="n"/>
+      <c r="E70" s="5" t="n"/>
+      <c r="F70" s="5" t="n"/>
     </row>
     <row r="71">
       <c r="B71" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Channel acct - ACV / account / yr</t>
-        </is>
-      </c>
-      <c r="C71" s="23">
-        <f>(1-Assumptions!$C$49)*(Assumptions!$C$66*Assumptions!$C$51)+Assumptions!$C$49*Assumptions!$C$52</f>
-        <v/>
+          <t>Manatal client base</t>
+        </is>
+      </c>
+      <c r="C71" s="20" t="n">
+        <v>10000</v>
       </c>
       <c r="D71" s="21" t="inlineStr">
         <is>
-          <t>$/yr</t>
-        </is>
-      </c>
-      <c r="E71" s="22" t="inlineStr"/>
+          <t>clients</t>
+        </is>
+      </c>
+      <c r="E71" s="22" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
       <c r="F71" s="21" t="inlineStr">
         <is>
-          <t>(1-ent%) x tests x blended price + ent% x flat fee.</t>
-        </is>
-      </c>
-    </row>
-    <row r="72" ht="20" customHeight="1">
-      <c r="B72" s="4" t="inlineStr">
-        <is>
-          <t>7.  SOM - Channel route (Manatal embedded)  [anchor 10,000+]</t>
-        </is>
-      </c>
-      <c r="C72" s="5" t="n"/>
-      <c r="D72" s="5" t="n"/>
-      <c r="E72" s="5" t="n"/>
-      <c r="F72" s="5" t="n"/>
+          <t>Anchor: embedded in Manatal, 10,000+ clients / 100+ countries.</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="B72" s="14" t="inlineStr">
+        <is>
+          <t>ICP-relevant share of Manatal base</t>
+        </is>
+      </c>
+      <c r="C72" s="26" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="D72" s="21" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E72" s="22" t="inlineStr"/>
+      <c r="F72" s="21" t="inlineStr">
+        <is>
+          <t>Manatal is a recruiter/agency ATS - most clients actively hire for roles Invirtus can assess.</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="B73" s="14" t="inlineStr">
         <is>
-          <t>Manatal client base</t>
-        </is>
-      </c>
-      <c r="C73" s="20" t="n">
-        <v>10000</v>
+          <t>Attach rate - year 1</t>
+        </is>
+      </c>
+      <c r="C73" s="24" t="n">
+        <v>0.02</v>
       </c>
       <c r="D73" s="21" t="inlineStr">
         <is>
-          <t>clients</t>
-        </is>
-      </c>
-      <c r="E73" s="22" t="inlineStr">
-        <is>
-          <t>S8</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E73" s="22" t="inlineStr"/>
       <c r="F73" s="21" t="inlineStr">
         <is>
-          <t>Anchor: embedded in Manatal, 10,000+ clients / 100+ countries.</t>
+          <t>Share of relevant Manatal clients activating Invirtus. Embedded distribution, low early activation.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="B74" s="14" t="inlineStr">
         <is>
-          <t>ICP-relevant share of Manatal base</t>
-        </is>
-      </c>
-      <c r="C74" s="26" t="n">
-        <v>0.45</v>
+          <t>Attach rate - year 2</t>
+        </is>
+      </c>
+      <c r="C74" s="24" t="n">
+        <v>0.05</v>
       </c>
       <c r="D74" s="21" t="inlineStr">
         <is>
@@ -2298,18 +2302,18 @@
       <c r="E74" s="22" t="inlineStr"/>
       <c r="F74" s="21" t="inlineStr">
         <is>
-          <t>Manatal is a recruiter/agency ATS - most clients actively hire for roles Invirtus can assess.</t>
+          <t>Ramp.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="B75" s="14" t="inlineStr">
         <is>
-          <t>Attach rate - year 1</t>
+          <t>Attach rate - year 3 (SOM)</t>
         </is>
       </c>
       <c r="C75" s="24" t="n">
-        <v>0.02</v>
+        <v>0.08</v>
       </c>
       <c r="D75" s="21" t="inlineStr">
         <is>
@@ -2319,117 +2323,117 @@
       <c r="E75" s="22" t="inlineStr"/>
       <c r="F75" s="21" t="inlineStr">
         <is>
-          <t>Share of relevant Manatal clients activating Invirtus. Embedded distribution, low early activation.</t>
+          <t>BIGGEST SOM DRIVER. Realistic embedded-tool attach, not best-in-class.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="B76" s="14" t="inlineStr">
         <is>
-          <t>Attach rate - year 2</t>
-        </is>
-      </c>
-      <c r="C76" s="24" t="n">
-        <v>0.05</v>
+          <t>Include 2nd ATS (Socium) in base?  (1/0)</t>
+        </is>
+      </c>
+      <c r="C76" s="30" t="n">
+        <v>0</v>
       </c>
       <c r="D76" s="21" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="E76" s="22" t="inlineStr"/>
       <c r="F76" s="21" t="inlineStr">
         <is>
-          <t>Ramp.</t>
+          <t>Held as UPSIDE until integration is real. Set 1 to include.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="B77" s="14" t="inlineStr">
         <is>
-          <t>Attach rate - year 3 (SOM)</t>
-        </is>
-      </c>
-      <c r="C77" s="24" t="n">
-        <v>0.08</v>
+          <t>Socium client base (upside)</t>
+        </is>
+      </c>
+      <c r="C77" s="20" t="n">
+        <v>3000</v>
       </c>
       <c r="D77" s="21" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E77" s="22" t="inlineStr"/>
+          <t>clients</t>
+        </is>
+      </c>
+      <c r="E77" s="22" t="inlineStr">
+        <is>
+          <t>S9</t>
+        </is>
+      </c>
       <c r="F77" s="21" t="inlineStr">
         <is>
-          <t>BIGGEST SOM DRIVER. Realistic embedded-tool attach, not best-in-class.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="B78" s="14" t="inlineStr">
-        <is>
-          <t>Include 2nd ATS (Socium) in base?  (1/0)</t>
-        </is>
-      </c>
-      <c r="C78" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D78" s="21" t="inlineStr">
-        <is>
-          <t>flag</t>
-        </is>
-      </c>
-      <c r="E78" s="22" t="inlineStr"/>
-      <c r="F78" s="21" t="inlineStr">
-        <is>
-          <t>Held as UPSIDE until integration is real. Set 1 to include.</t>
-        </is>
-      </c>
+          <t>Upside only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="20" customHeight="1">
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>8.  SOM - Direct route (self-serve + sales-led)</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="n"/>
+      <c r="D78" s="5" t="n"/>
+      <c r="E78" s="5" t="n"/>
+      <c r="F78" s="5" t="n"/>
     </row>
     <row r="79">
       <c r="B79" s="14" t="inlineStr">
         <is>
-          <t>Socium client base (upside)</t>
-        </is>
-      </c>
-      <c r="C79" s="20" t="n">
-        <v>3000</v>
+          <t>3-yr penetration of serviceable SAM accounts</t>
+        </is>
+      </c>
+      <c r="C79" s="24" t="n">
+        <v>0.008</v>
       </c>
       <c r="D79" s="21" t="inlineStr">
         <is>
-          <t>clients</t>
-        </is>
-      </c>
-      <c r="E79" s="22" t="inlineStr">
-        <is>
-          <t>S9</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E79" s="22" t="inlineStr"/>
       <c r="F79" s="21" t="inlineStr">
         <is>
-          <t>Upside only.</t>
-        </is>
-      </c>
-    </row>
-    <row r="80" ht="20" customHeight="1">
-      <c r="B80" s="4" t="inlineStr">
-        <is>
-          <t>8.  SOM - Direct route (self-serve + sales-led)</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="n"/>
-      <c r="D80" s="5" t="n"/>
-      <c r="E80" s="5" t="n"/>
-      <c r="F80" s="5" t="n"/>
+          <t>Direct capture is gated by low trial-to-paid; a pre-seed wins only a thin slice of the large serviceable base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="B80" s="14" t="inlineStr">
+        <is>
+          <t>Monthly website traffic</t>
+        </is>
+      </c>
+      <c r="C80" s="20" t="n">
+        <v>8000</v>
+      </c>
+      <c r="D80" s="21" t="inlineStr">
+        <is>
+          <t>visits/mo</t>
+        </is>
+      </c>
+      <c r="E80" s="22" t="inlineStr"/>
+      <c r="F80" s="21" t="inlineStr">
+        <is>
+          <t>Self-serve funnel cross-check input (year-3 run-rate).</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="B81" s="14" t="inlineStr">
         <is>
-          <t>3-yr penetration of serviceable SAM accounts</t>
+          <t>Visit -&gt; free-trial conversion</t>
         </is>
       </c>
       <c r="C81" s="24" t="n">
-        <v>0.008</v>
+        <v>0.03</v>
       </c>
       <c r="D81" s="21" t="inlineStr">
         <is>
@@ -2437,58 +2441,52 @@
         </is>
       </c>
       <c r="E81" s="22" t="inlineStr"/>
-      <c r="F81" s="21" t="inlineStr">
-        <is>
-          <t>Direct capture is gated by low trial-to-paid; a pre-seed wins only a thin slice of the large serviceable base.</t>
-        </is>
-      </c>
+      <c r="F81" s="21" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="B82" s="14" t="inlineStr">
         <is>
-          <t>Monthly website traffic</t>
-        </is>
-      </c>
-      <c r="C82" s="20" t="n">
-        <v>8000</v>
+          <t>Trial -&gt; paid conversion</t>
+        </is>
+      </c>
+      <c r="C82" s="24" t="n">
+        <v>0.05</v>
       </c>
       <c r="D82" s="21" t="inlineStr">
         <is>
-          <t>visits/mo</t>
-        </is>
-      </c>
-      <c r="E82" s="22" t="inlineStr"/>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E82" s="22" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
       <c r="F82" s="21" t="inlineStr">
         <is>
-          <t>Self-serve funnel cross-check input (year-3 run-rate).</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="B83" s="14" t="inlineStr">
-        <is>
-          <t>Visit -&gt; free-trial conversion</t>
-        </is>
-      </c>
-      <c r="C83" s="24" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="D83" s="21" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E83" s="22" t="inlineStr"/>
-      <c r="F83" s="21" t="inlineStr"/>
+          <t>Currently LOW - do NOT assume best-in-class. Flagged in GTM notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="20" customHeight="1">
+      <c r="B83" s="4" t="inlineStr">
+        <is>
+          <t>9.  Retention &amp; global scope</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="n"/>
+      <c r="D83" s="5" t="n"/>
+      <c r="E83" s="5" t="n"/>
+      <c r="F83" s="5" t="n"/>
     </row>
     <row r="84">
       <c r="B84" s="14" t="inlineStr">
         <is>
-          <t>Trial -&gt; paid conversion</t>
+          <t>Steady-state annual retention</t>
         </is>
       </c>
       <c r="C84" s="24" t="n">
-        <v>0.05</v>
+        <v>0.9</v>
       </c>
       <c r="D84" s="21" t="inlineStr">
         <is>
@@ -2502,140 +2500,104 @@
       </c>
       <c r="F84" s="21" t="inlineStr">
         <is>
-          <t>Currently LOW - do NOT assume best-in-class. Flagged in GTM notes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="20" customHeight="1">
-      <c r="B85" s="4" t="inlineStr">
-        <is>
-          <t>9.  Retention &amp; global scope</t>
-        </is>
-      </c>
-      <c r="C85" s="5" t="n"/>
-      <c r="D85" s="5" t="n"/>
-      <c r="E85" s="5" t="n"/>
-      <c r="F85" s="5" t="n"/>
-    </row>
-    <row r="86">
-      <c r="B86" s="14" t="inlineStr">
-        <is>
-          <t>Steady-state annual retention</t>
-        </is>
-      </c>
-      <c r="C86" s="24" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="D86" s="21" t="inlineStr">
+          <t>Finalized BP assumes 7% gross churn (93% retention); held slightly conservative at 90% for the SOM. 100% to date on a tiny base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="B85" s="14" t="inlineStr">
+        <is>
+          <t>Focus-6 share of global addressable universe</t>
+        </is>
+      </c>
+      <c r="C85" s="24" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="D85" s="21" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E86" s="22" t="inlineStr">
-        <is>
-          <t>S8</t>
-        </is>
-      </c>
-      <c r="F86" s="21" t="inlineStr">
-        <is>
-          <t>100% to date on 3 accounts; model realistic steady-state, not 100%.</t>
-        </is>
-      </c>
+      <c r="E85" s="22" t="inlineStr"/>
+      <c r="F85" s="21" t="inlineStr">
+        <is>
+          <t>Focus-6 as % of all geos where product works. Grosses SAM up to TAM. US/India/rest-EU dominate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="20" customHeight="1">
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>10. Value delivered  (cost-of-bad-hire anchor)</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="n"/>
+      <c r="D86" s="5" t="n"/>
+      <c r="E86" s="5" t="n"/>
+      <c r="F86" s="5" t="n"/>
     </row>
     <row r="87">
       <c r="B87" s="14" t="inlineStr">
         <is>
-          <t>Focus-6 share of global addressable universe</t>
-        </is>
-      </c>
-      <c r="C87" s="24" t="n">
-        <v>0.12</v>
+          <t>Cost of a bad hire</t>
+        </is>
+      </c>
+      <c r="C87" s="20" t="n">
+        <v>150000</v>
       </c>
       <c r="D87" s="21" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E87" s="22" t="inlineStr"/>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="E87" s="22" t="inlineStr">
+        <is>
+          <t>S8</t>
+        </is>
+      </c>
       <c r="F87" s="21" t="inlineStr">
         <is>
-          <t>Focus-6 as % of all geos where product works. Grosses SAM up to TAM. US/India/rest-EU dominate.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="20" customHeight="1">
-      <c r="B88" s="4" t="inlineStr">
-        <is>
-          <t>10. Value delivered  (cost-of-bad-hire anchor)</t>
-        </is>
-      </c>
-      <c r="C88" s="5" t="n"/>
-      <c r="D88" s="5" t="n"/>
-      <c r="E88" s="5" t="n"/>
-      <c r="F88" s="5" t="n"/>
+          <t>Core value anchor used across sales &amp; fundraising.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="14" t="inlineStr">
+        <is>
+          <t>Tests run per hire placed</t>
+        </is>
+      </c>
+      <c r="C88" s="20" t="n">
+        <v>6</v>
+      </c>
+      <c r="D88" s="21" t="inlineStr">
+        <is>
+          <t>tests</t>
+        </is>
+      </c>
+      <c r="E88" s="22" t="inlineStr"/>
+      <c r="F88" s="21" t="inlineStr">
+        <is>
+          <t>Candidates assessed per filled role (1 hire/role).</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="B89" s="14" t="inlineStr">
         <is>
-          <t>Cost of a bad hire</t>
-        </is>
-      </c>
-      <c r="C89" s="20" t="n">
-        <v>150000</v>
+          <t>Bad-hire rate reduction from structured eval</t>
+        </is>
+      </c>
+      <c r="C89" s="26" t="n">
+        <v>0.2</v>
       </c>
       <c r="D89" s="21" t="inlineStr">
         <is>
-          <t>$</t>
-        </is>
-      </c>
-      <c r="E89" s="22" t="inlineStr">
-        <is>
-          <t>S8</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E89" s="22" t="inlineStr"/>
       <c r="F89" s="21" t="inlineStr">
-        <is>
-          <t>Core value anchor used across sales &amp; fundraising.</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="B90" s="14" t="inlineStr">
-        <is>
-          <t>Tests run per hire placed</t>
-        </is>
-      </c>
-      <c r="C90" s="20" t="n">
-        <v>6</v>
-      </c>
-      <c r="D90" s="21" t="inlineStr">
-        <is>
-          <t>tests</t>
-        </is>
-      </c>
-      <c r="E90" s="22" t="inlineStr"/>
-      <c r="F90" s="21" t="inlineStr">
-        <is>
-          <t>Candidates assessed per filled role (1 hire/role).</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="B91" s="14" t="inlineStr">
-        <is>
-          <t>Bad-hire rate reduction from structured eval</t>
-        </is>
-      </c>
-      <c r="C91" s="26" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D91" s="21" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E91" s="22" t="inlineStr"/>
-      <c r="F91" s="21" t="inlineStr">
         <is>
           <t>Assumed share of bad-hire cost avoided via better screening.</t>
         </is>
@@ -2751,11 +2713,11 @@
         <v/>
       </c>
       <c r="F6" s="32">
-        <f>Assumptions!$C$57</f>
+        <f>Assumptions!$C$55</f>
         <v/>
       </c>
       <c r="G6" s="32">
-        <f>Assumptions!$C$68</f>
+        <f>Assumptions!$C$66</f>
         <v/>
       </c>
       <c r="H6" s="32">
@@ -2782,11 +2744,11 @@
         <v/>
       </c>
       <c r="F7" s="32">
-        <f>Assumptions!$C$60</f>
+        <f>Assumptions!$C$58</f>
         <v/>
       </c>
       <c r="G7" s="32">
-        <f>Assumptions!$C$69</f>
+        <f>Assumptions!$C$67</f>
         <v/>
       </c>
       <c r="H7" s="32">
@@ -2813,11 +2775,11 @@
         <v/>
       </c>
       <c r="F8" s="32">
-        <f>Assumptions!$C$63</f>
+        <f>Assumptions!$C$61</f>
         <v/>
       </c>
       <c r="G8" s="32">
-        <f>Assumptions!$C$70</f>
+        <f>Assumptions!$C$68</f>
         <v/>
       </c>
       <c r="H8" s="32">
@@ -2899,7 +2861,7 @@
         </is>
       </c>
       <c r="C14" s="32">
-        <f>Assumptions!$C$28/Assumptions!$C$87</f>
+        <f>Assumptions!$C$28/Assumptions!$C$85</f>
         <v/>
       </c>
       <c r="D14" s="33">
@@ -2911,7 +2873,7 @@
         <v/>
       </c>
       <c r="F14" s="32">
-        <f>Assumptions!$C$68</f>
+        <f>Assumptions!$C$66</f>
         <v/>
       </c>
       <c r="G14" s="32">
@@ -2926,7 +2888,7 @@
         </is>
       </c>
       <c r="C15" s="32">
-        <f>Assumptions!$C$29/Assumptions!$C$87</f>
+        <f>Assumptions!$C$29/Assumptions!$C$85</f>
         <v/>
       </c>
       <c r="D15" s="33">
@@ -2938,7 +2900,7 @@
         <v/>
       </c>
       <c r="F15" s="32">
-        <f>Assumptions!$C$69</f>
+        <f>Assumptions!$C$67</f>
         <v/>
       </c>
       <c r="G15" s="32">
@@ -2953,7 +2915,7 @@
         </is>
       </c>
       <c r="C16" s="32">
-        <f>Assumptions!$C$30/Assumptions!$C$87</f>
+        <f>Assumptions!$C$30/Assumptions!$C$85</f>
         <v/>
       </c>
       <c r="D16" s="33">
@@ -2965,7 +2927,7 @@
         <v/>
       </c>
       <c r="F16" s="32">
-        <f>Assumptions!$C$70</f>
+        <f>Assumptions!$C$68</f>
         <v/>
       </c>
       <c r="G16" s="32">
@@ -3026,15 +2988,15 @@
         </is>
       </c>
       <c r="C21" s="32">
-        <f>(Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74</f>
+        <f>(Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72</f>
         <v/>
       </c>
       <c r="D21" s="32">
-        <f>(Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74</f>
+        <f>(Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72</f>
         <v/>
       </c>
       <c r="E21" s="32">
-        <f>(Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74</f>
+        <f>(Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72</f>
         <v/>
       </c>
     </row>
@@ -3045,15 +3007,15 @@
         </is>
       </c>
       <c r="C22" s="33">
+        <f>Assumptions!$C$73</f>
+        <v/>
+      </c>
+      <c r="D22" s="33">
+        <f>Assumptions!$C$74</f>
+        <v/>
+      </c>
+      <c r="E22" s="33">
         <f>Assumptions!$C$75</f>
-        <v/>
-      </c>
-      <c r="D22" s="33">
-        <f>Assumptions!$C$76</f>
-        <v/>
-      </c>
-      <c r="E22" s="33">
-        <f>Assumptions!$C$77</f>
         <v/>
       </c>
     </row>
@@ -3083,15 +3045,15 @@
         </is>
       </c>
       <c r="C24" s="36">
-        <f>C23*Assumptions!$C$71*Assumptions!$C$86</f>
+        <f>C23*Assumptions!$C$69*Assumptions!$C$84</f>
         <v/>
       </c>
       <c r="D24" s="36">
-        <f>D23*Assumptions!$C$71*Assumptions!$C$86</f>
+        <f>D23*Assumptions!$C$69*Assumptions!$C$84</f>
         <v/>
       </c>
       <c r="E24" s="36">
-        <f>E23*Assumptions!$C$71*Assumptions!$C$86</f>
+        <f>E23*Assumptions!$C$69*Assumptions!$C$84</f>
         <v/>
       </c>
     </row>
@@ -3127,7 +3089,7 @@
         </is>
       </c>
       <c r="E28" s="33">
-        <f>Assumptions!$C$81</f>
+        <f>Assumptions!$C$79</f>
         <v/>
       </c>
     </row>
@@ -3149,7 +3111,7 @@
         </is>
       </c>
       <c r="E30" s="36">
-        <f>Build!$H$9*E28*Assumptions!$C$86</f>
+        <f>Build!$H$9*E28*Assumptions!$C$84</f>
         <v/>
       </c>
     </row>
@@ -3160,7 +3122,7 @@
         </is>
       </c>
       <c r="E31" s="37">
-        <f>Assumptions!$C$82*12*Assumptions!$C$83*Assumptions!$C$84</f>
+        <f>Assumptions!$C$80*12*Assumptions!$C$81*Assumptions!$C$82</f>
         <v/>
       </c>
     </row>
@@ -3231,19 +3193,19 @@
         <v/>
       </c>
       <c r="D37" s="32">
-        <f>C37*Assumptions!$C$66</f>
+        <f>C37*Assumptions!$C$64</f>
         <v/>
       </c>
       <c r="E37" s="32">
-        <f>D37/Assumptions!$C$90</f>
+        <f>D37/Assumptions!$C$88</f>
         <v/>
       </c>
       <c r="F37" s="32">
-        <f>E37*Assumptions!$C$89</f>
+        <f>E37*Assumptions!$C$87</f>
         <v/>
       </c>
       <c r="G37" s="32">
-        <f>F37*Assumptions!$C$91</f>
+        <f>F37*Assumptions!$C$89</f>
         <v/>
       </c>
     </row>
@@ -3330,23 +3292,23 @@
         <v>100</v>
       </c>
       <c r="C7" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B7*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B7*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D7" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B7*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B7*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E7" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B7*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B7*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F7" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B7*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B7*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G7" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B7*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B7*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3355,23 +3317,23 @@
         <v>150</v>
       </c>
       <c r="C8" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B8*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B8*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D8" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B8*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B8*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E8" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B8*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B8*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F8" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B8*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B8*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G8" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B8*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B8*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3380,23 +3342,23 @@
         <v>200</v>
       </c>
       <c r="C9" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B9*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B9*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D9" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B9*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B9*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E9" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B9*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B9*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F9" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B9*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B9*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G9" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B9*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B9*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3405,23 +3367,23 @@
         <v>250</v>
       </c>
       <c r="C10" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B10*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B10*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D10" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B10*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B10*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E10" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B10*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B10*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F10" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B10*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B10*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G10" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B10*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B10*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3430,23 +3392,23 @@
         <v>300</v>
       </c>
       <c r="C11" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B11*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B11*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*C$6+Assumptions!$C$46*C$6*(1-Assumptions!$C$37)+Assumptions!$C$47*C$6*(1-Assumptions!$C$38)+Assumptions!$C$48*C$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D11" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B11*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B11*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*D$6+Assumptions!$C$46*D$6*(1-Assumptions!$C$37)+Assumptions!$C$47*D$6*(1-Assumptions!$C$38)+Assumptions!$C$48*D$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E11" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B11*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B11*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*E$6+Assumptions!$C$46*E$6*(1-Assumptions!$C$37)+Assumptions!$C$47*E$6*(1-Assumptions!$C$38)+Assumptions!$C$48*E$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F11" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B11*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B11*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*F$6+Assumptions!$C$46*F$6*(1-Assumptions!$C$37)+Assumptions!$C$47*F$6*(1-Assumptions!$C$38)+Assumptions!$C$48*F$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G11" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*($B11*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*($B11*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*G$6+Assumptions!$C$46*G$6*(1-Assumptions!$C$37)+Assumptions!$C$47*G$6*(1-Assumptions!$C$38)+Assumptions!$C$48*G$6*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3484,23 +3446,23 @@
         <v>0.04</v>
       </c>
       <c r="C15" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B15*((1-Assumptions!$C$49)*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B15*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D15" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B15*((1-Assumptions!$C$49)*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B15*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E15" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B15*((1-Assumptions!$C$49)*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B15*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F15" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B15*((1-Assumptions!$C$49)*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B15*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G15" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B15*((1-Assumptions!$C$49)*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B15*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3509,23 +3471,23 @@
         <v>0.06</v>
       </c>
       <c r="C16" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B16*((1-Assumptions!$C$49)*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B16*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D16" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B16*((1-Assumptions!$C$49)*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B16*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E16" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B16*((1-Assumptions!$C$49)*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B16*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F16" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B16*((1-Assumptions!$C$49)*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B16*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G16" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B16*((1-Assumptions!$C$49)*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B16*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3534,23 +3496,23 @@
         <v>0.08</v>
       </c>
       <c r="C17" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B17*((1-Assumptions!$C$49)*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B17*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D17" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B17*((1-Assumptions!$C$49)*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B17*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E17" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B17*((1-Assumptions!$C$49)*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B17*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F17" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B17*((1-Assumptions!$C$49)*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B17*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G17" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B17*((1-Assumptions!$C$49)*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B17*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3559,23 +3521,23 @@
         <v>0.1</v>
       </c>
       <c r="C18" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B18*((1-Assumptions!$C$49)*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B18*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D18" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B18*((1-Assumptions!$C$49)*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B18*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E18" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B18*((1-Assumptions!$C$49)*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B18*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F18" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B18*((1-Assumptions!$C$49)*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B18*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G18" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B18*((1-Assumptions!$C$49)*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B18*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3584,23 +3546,23 @@
         <v>0.12</v>
       </c>
       <c r="C19" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B19*((1-Assumptions!$C$49)*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B19*(C$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D19" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B19*((1-Assumptions!$C$49)*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B19*(D$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E19" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B19*((1-Assumptions!$C$49)*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B19*(E$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="F19" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B19*((1-Assumptions!$C$49)*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B19*(F$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="G19" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*$B19*((1-Assumptions!$C$49)*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*$B19*(G$14*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3640,15 +3602,15 @@
         </is>
       </c>
       <c r="C24" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*0.04*((1-Assumptions!$C$49)*(Assumptions!$C$66*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*0.04*(Assumptions!$C$64*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D24" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*(Assumptions!$C$66*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*(Assumptions!$C$64*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E24" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*0.12*((1-Assumptions!$C$49)*(Assumptions!$C$66*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*0.12*(Assumptions!$C$64*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3659,34 +3621,34 @@
         </is>
       </c>
       <c r="C25" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*(100*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*(100*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D25" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*(Assumptions!$C$66*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*(Assumptions!$C$64*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E25" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*(300*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*(300*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="12" t="inlineStr">
         <is>
-          <t>PAYG price/test ($10 / $15 / $20)</t>
+          <t>PAYG price/test ($10 / base $14 / $20)</t>
         </is>
       </c>
       <c r="C26" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*(Assumptions!$C$66*((Assumptions!$C$45*10+Assumptions!$C$46*10*(1-Assumptions!$C$37)+Assumptions!$C$47*10*(1-Assumptions!$C$38)+Assumptions!$C$48*10*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*10+Assumptions!$C$46*10*(1-Assumptions!$C$37)+Assumptions!$C$47*10*(1-Assumptions!$C$38)+Assumptions!$C$48*10*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*10+Assumptions!$C$46*10*(1-Assumptions!$C$37)+Assumptions!$C$47*10*(1-Assumptions!$C$38)+Assumptions!$C$48*10*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*10+Assumptions!$C$46*10*(1-Assumptions!$C$37)+Assumptions!$C$47*10*(1-Assumptions!$C$38)+Assumptions!$C$48*10*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*(Assumptions!$C$64*((Assumptions!$C$45*10+Assumptions!$C$46*10*(1-Assumptions!$C$37)+Assumptions!$C$47*10*(1-Assumptions!$C$38)+Assumptions!$C$48*10*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*10+Assumptions!$C$46*10*(1-Assumptions!$C$37)+Assumptions!$C$47*10*(1-Assumptions!$C$38)+Assumptions!$C$48*10*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*10+Assumptions!$C$46*10*(1-Assumptions!$C$37)+Assumptions!$C$47*10*(1-Assumptions!$C$38)+Assumptions!$C$48*10*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*10+Assumptions!$C$46*10*(1-Assumptions!$C$37)+Assumptions!$C$47*10*(1-Assumptions!$C$38)+Assumptions!$C$48*10*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="D26" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*(Assumptions!$C$66*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*(Assumptions!$C$64*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*Assumptions!$C$36+Assumptions!$C$46*Assumptions!$C$36*(1-Assumptions!$C$37)+Assumptions!$C$47*Assumptions!$C$36*(1-Assumptions!$C$38)+Assumptions!$C$48*Assumptions!$C$36*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
       <c r="E26" s="42">
-        <f>((Assumptions!$C$73+Assumptions!$C$78*Assumptions!$C$79)*Assumptions!$C$74)*Assumptions!$C$77*((1-Assumptions!$C$49)*(Assumptions!$C$66*((Assumptions!$C$45*20+Assumptions!$C$46*20*(1-Assumptions!$C$37)+Assumptions!$C$47*20*(1-Assumptions!$C$38)+Assumptions!$C$48*20*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)*Assumptions!$C$86+(((Assumptions!$C$28*Assumptions!$C$32*((1-Assumptions!$C$49)*((Assumptions!$C$55*Assumptions!$C$56*Assumptions!$C$54)*((Assumptions!$C$45*20+Assumptions!$C$46*20*(1-Assumptions!$C$37)+Assumptions!$C$47*20*(1-Assumptions!$C$38)+Assumptions!$C$48*20*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$29*Assumptions!$C$33*((1-Assumptions!$C$49)*((Assumptions!$C$58*Assumptions!$C$59*Assumptions!$C$54)*((Assumptions!$C$45*20+Assumptions!$C$46*20*(1-Assumptions!$C$37)+Assumptions!$C$47*20*(1-Assumptions!$C$38)+Assumptions!$C$48*20*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52))+(Assumptions!$C$30*Assumptions!$C$34*((1-Assumptions!$C$49)*((Assumptions!$C$61*Assumptions!$C$62*Assumptions!$C$54)*((Assumptions!$C$45*20+Assumptions!$C$46*20*(1-Assumptions!$C$37)+Assumptions!$C$47*20*(1-Assumptions!$C$38)+Assumptions!$C$48*20*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))+Assumptions!$C$49*Assumptions!$C$52)))*Assumptions!$C$81*Assumptions!$C$86)</f>
+        <f>((Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72)*Assumptions!$C$75*(Assumptions!$C$64*((Assumptions!$C$45*20+Assumptions!$C$46*20*(1-Assumptions!$C$37)+Assumptions!$C$47*20*(1-Assumptions!$C$38)+Assumptions!$C$48*20*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))*Assumptions!$C$84+(((Assumptions!$C$28*Assumptions!$C$32*((Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52)*((Assumptions!$C$45*20+Assumptions!$C$46*20*(1-Assumptions!$C$37)+Assumptions!$C$47*20*(1-Assumptions!$C$38)+Assumptions!$C$48*20*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$29*Assumptions!$C$33*((Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52)*((Assumptions!$C$45*20+Assumptions!$C$46*20*(1-Assumptions!$C$37)+Assumptions!$C$47*20*(1-Assumptions!$C$38)+Assumptions!$C$48*20*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48))))+(Assumptions!$C$30*Assumptions!$C$34*((Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52)*((Assumptions!$C$45*20+Assumptions!$C$46*20*(1-Assumptions!$C$37)+Assumptions!$C$47*20*(1-Assumptions!$C$38)+Assumptions!$C$48*20*(1-Assumptions!$C$39))/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)))))*Assumptions!$C$79*Assumptions!$C$84)</f>
         <v/>
       </c>
     </row>
@@ -3962,22 +3924,22 @@
       </c>
       <c r="C12" s="46" t="inlineStr">
         <is>
-          <t>Pricing benchmark ($15/test, ent. fee)</t>
+          <t>Pricing: $14/test + packs (finalized BP); benchmarked</t>
         </is>
       </c>
       <c r="D12" s="46" t="inlineStr">
         <is>
-          <t>TestGorilla; TestDome; Adaface; HackerRank; Codility pricing</t>
+          <t>Invirtus finalized BP (Aida); TestGorilla; TestDome; Adaface; HackerRank pricing</t>
         </is>
       </c>
       <c r="E12" s="47" t="inlineStr">
         <is>
-          <t>testgorilla.com/pricing ; testdome.com/pricing ; adaface.com/pricing</t>
+          <t>Invirtus_business_plan.xlsx ; testgorilla.com/pricing ; testdome.com/pricing ; adaface.com/pricing</t>
         </is>
       </c>
       <c r="F12" s="48" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="G12" s="48" t="inlineStr">

</xml_diff>

<commit_message>
Reframe as Revenue Potential and add talent-DB as a second stream
- Reframed the headline from "Market Sizing / TAM-SAM-SOM" to "Revenue
  Potential" with plain-English tiers (Full opportunity / Serviceable today /
  3-year reachable), keeping TAM/SAM/SOM tags for investor familiarity.
- Added talent-DB monetization as a second revenue stream, modeled as in the
  finalized BP: DB revenue = tests run x % profiles sourced from own DB (mature
  30%) x $30/profile. New Build block D shows both streams + total per tier;
  Cover cards now show total revenue potential with a stream split.

Totals (assessments + DB): Full opportunity ~$1.11B, Serviceable ~$133M,
3-year reachable ~$2.34M ($1.34M assessments + $0.99M DB). 0 formula errors.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RsCNYhV2EbucLSqzkWAFLN
</commit_message>
<xml_diff>
--- a/Invirtus_Market_Sizing.xlsx
+++ b/Invirtus_Market_Sizing.xlsx
@@ -191,6 +191,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -237,7 +238,6 @@
     </xf>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -627,7 +627,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E26"/>
+  <dimension ref="B2:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -648,7 +648,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Bottoms-Up Market Sizing  -  TAM / SAM / SOM</t>
+          <t>Bottoms-Up Revenue Potential  (two streams; TAM / SAM / SOM equivalents)</t>
         </is>
       </c>
     </row>
@@ -672,7 +672,7 @@
     <row r="7">
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Lead with SOM. Reachable 3-year revenue is driven first by the Manatal channel (embedded attach ~56% of SOM), then self-serve. The single biggest assumption is the Year-3 channel attach rate on the ICP-relevant Manatal base (Assumptions sec. 7). Tests/account and the $14 PAYG price are the next two swing factors (see Sensitivity).</t>
+          <t>Lead with the 3-year reachable number. It runs on two streams - assessment packs plus talent-DB monetization - and is driven first by the Manatal channel (embedded attach ~59% of the assessment line), then self-serve. The single biggest assumption is the Year-3 channel attach rate on the ICP-relevant Manatal base (Assumptions sec. 7); tests/account and the $14 PAYG price are the next two swing factors (see Sensitivity).</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -694,129 +694,169 @@
     <row r="11">
       <c r="B11" s="8" t="inlineStr">
         <is>
-          <t>TAM</t>
+          <t>FULL OPPORTUNITY</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
         <is>
-          <t>SAM</t>
+          <t>SERVICEABLE TODAY</t>
         </is>
       </c>
       <c r="D11" s="8" t="inlineStr">
         <is>
-          <t>SOM (Yr 3)</t>
+          <t>3-YEAR REACHABLE</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="9">
-        <f>Build!$G$17</f>
-        <v/>
-      </c>
-      <c r="C12" s="9">
-        <f>Build!$H$9</f>
+        <f>Build!$F$37</f>
+        <v/>
+      </c>
+      <c r="C12" s="10">
+        <f>Build!$F$38</f>
         <v/>
       </c>
       <c r="D12" s="10">
-        <f>Build!$E$33</f>
+        <f>Build!$F$39</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Global prize, full ACV</t>
+          <t>(TAM) all geos | 2 streams</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Focus-6, serviceable today</t>
+          <t>(SAM) focus-6 | serviceable</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Channel + direct, retention-adj</t>
+          <t>(SOM) channel+direct | 3-yr</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>SOM split</t>
+          <t>3-yr reachable - by revenue stream</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="12" t="inlineStr">
         <is>
-          <t>Channel (Manatal)</t>
+          <t>Assessment packs</t>
         </is>
       </c>
       <c r="C16" s="13">
-        <f>Build!$E$24</f>
+        <f>Build!$C$39</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="12" t="inlineStr">
         <is>
+          <t>Talent-DB monetization</t>
+        </is>
+      </c>
+      <c r="C17" s="13">
+        <f>Build!$E$39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="14" t="inlineStr">
+        <is>
+          <t>Total revenue potential</t>
+        </is>
+      </c>
+      <c r="C18" s="13">
+        <f>Build!$F$39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>3-yr reachable - assessments by route</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Channel (Manatal)</t>
+        </is>
+      </c>
+      <c r="C21" s="13">
+        <f>Build!$E$24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="12" t="inlineStr">
+        <is>
           <t>Direct (self-serve + sales)</t>
         </is>
       </c>
-      <c r="C17" s="13">
+      <c r="C22" s="13">
         <f>Build!$E$30</f>
         <v/>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="11" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>How to read this model</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="14" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t>1.  Every blue cell on Assumptions is an editable input; black cells are formulas with no hardcodes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>2.  Build derives SAM bottoms-up (entities x %fit x tests/yr x net $/test), grosses up to TAM, and</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     captures SOM via two real routes: the Manatal channel and direct self-serve/sales.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>3.  Sensitivity flexes the three inputs that move SOM most. Sources lists every researched figure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>4.  Value-delivered read ties tests -&gt; hires -&gt; the $150k cost-of-bad-hire anchor.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="15" t="inlineStr">
         <is>
+          <t>2.  Build derives SAM bottoms-up (entities x %fit x tests/yr x net $/test), grosses up to TAM, and</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     captures SOM via two real routes: the Manatal channel and direct self-serve/sales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="15" t="inlineStr">
+        <is>
+          <t>3.  Sensitivity flexes the three inputs that move SOM most. Sources lists every researched figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>4.  Value-delivered read ties tests -&gt; hires -&gt; the $150k cost-of-bad-hire anchor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="16" t="inlineStr">
+        <is>
           <t>Input (editable)</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C31" s="12" t="inlineStr">
         <is>
           <t>Formula (calc)</t>
         </is>
@@ -824,12 +864,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="B23:E23"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="B24:E24"/>
-    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="B26:E26"/>
+    <mergeCell ref="B27:E27"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B25:E25"/>
     <mergeCell ref="B7:E9"/>
-    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B28:E28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -841,7 +881,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:F89"/>
+  <dimension ref="B1:F92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -853,41 +893,41 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="16" t="inlineStr">
+      <c r="B1" s="17" t="inlineStr">
         <is>
           <t>INVIRTUS  -  Assumptions</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="17" t="inlineStr">
+      <c r="B2" s="18" t="inlineStr">
         <is>
           <t>All blue cells are editable inputs. Black cells are formulas. Col E = source key (see Sources tab). Currency = USD.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="18" t="inlineStr">
+      <c r="B4" s="19" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>Src</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>Logic / flag</t>
         </is>
@@ -905,560 +945,560 @@
       <c r="F5" s="5" t="n"/>
     </row>
     <row r="6">
-      <c r="B6" s="18" t="inlineStr">
+      <c r="B6" s="19" t="inlineStr">
         <is>
           <t>Tech-focused recruiting agencies</t>
         </is>
       </c>
-      <c r="C6" s="19" t="n"/>
-      <c r="D6" s="19" t="n"/>
-      <c r="E6" s="19" t="n"/>
-      <c r="F6" s="19" t="n"/>
+      <c r="C6" s="20" t="n"/>
+      <c r="D6" s="20" t="n"/>
+      <c r="E6" s="20" t="n"/>
+      <c r="F6" s="20" t="n"/>
     </row>
     <row r="7">
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   France</t>
         </is>
       </c>
-      <c r="C7" s="20" t="n">
+      <c r="C7" s="21" t="n">
         <v>500</v>
       </c>
-      <c r="D7" s="21" t="inlineStr">
+      <c r="D7" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E7" s="22" t="inlineStr">
+      <c r="E7" s="23" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="F7" s="21" t="inlineStr">
+      <c r="F7" s="22" t="inlineStr">
         <is>
           <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   UK</t>
         </is>
       </c>
-      <c r="C8" s="20" t="n">
+      <c r="C8" s="21" t="n">
         <v>3500</v>
       </c>
-      <c r="D8" s="21" t="inlineStr">
+      <c r="D8" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E8" s="22" t="inlineStr">
+      <c r="E8" s="23" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="F8" s="21" t="inlineStr">
+      <c r="F8" s="22" t="inlineStr">
         <is>
           <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   UAE</t>
         </is>
       </c>
-      <c r="C9" s="20" t="n">
+      <c r="C9" s="21" t="n">
         <v>100</v>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E9" s="22" t="inlineStr">
+      <c r="E9" s="23" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="F9" s="21" t="inlineStr">
+      <c r="F9" s="22" t="inlineStr">
         <is>
           <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Morocco</t>
         </is>
       </c>
-      <c r="C10" s="20" t="n">
+      <c r="C10" s="21" t="n">
         <v>45</v>
       </c>
-      <c r="D10" s="21" t="inlineStr">
+      <c r="D10" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E10" s="22" t="inlineStr">
+      <c r="E10" s="23" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="F10" s="21" t="inlineStr">
+      <c r="F10" s="22" t="inlineStr">
         <is>
           <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   KSA</t>
         </is>
       </c>
-      <c r="C11" s="20" t="n">
+      <c r="C11" s="21" t="n">
         <v>50</v>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E11" s="22" t="inlineStr">
+      <c r="E11" s="23" t="inlineStr">
         <is>
           <t>S5</t>
         </is>
       </c>
-      <c r="F11" s="21" t="inlineStr">
+      <c r="F11" s="22" t="inlineStr">
         <is>
           <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Egypt</t>
         </is>
       </c>
-      <c r="C12" s="20" t="n">
+      <c r="C12" s="21" t="n">
         <v>60</v>
       </c>
-      <c r="D12" s="21" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E12" s="22" t="inlineStr">
+      <c r="E12" s="23" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="F12" s="21" t="inlineStr">
+      <c r="F12" s="22" t="inlineStr">
         <is>
           <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="18" t="inlineStr">
+      <c r="B13" s="19" t="inlineStr">
         <is>
           <t>Engineering-heavy firms (tech/software/ICT cos.)</t>
         </is>
       </c>
-      <c r="C13" s="19" t="n"/>
-      <c r="D13" s="19" t="n"/>
-      <c r="E13" s="19" t="n"/>
-      <c r="F13" s="19" t="n"/>
+      <c r="C13" s="20" t="n"/>
+      <c r="D13" s="20" t="n"/>
+      <c r="E13" s="20" t="n"/>
+      <c r="F13" s="20" t="n"/>
     </row>
     <row r="14">
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   France</t>
         </is>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="21" t="n">
         <v>95000</v>
       </c>
-      <c r="D14" s="21" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E14" s="22" t="inlineStr">
+      <c r="E14" s="23" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="F14" s="21" t="inlineStr">
+      <c r="F14" s="22" t="inlineStr">
         <is>
           <t>Tech/software/ICT companies that hire engineers in-house.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   UK</t>
         </is>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="21" t="n">
         <v>107000</v>
       </c>
-      <c r="D15" s="21" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E15" s="22" t="inlineStr">
+      <c r="E15" s="23" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="F15" s="21" t="inlineStr">
+      <c r="F15" s="22" t="inlineStr">
         <is>
           <t>Tech/software/ICT companies that hire engineers in-house.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="14" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   UAE</t>
         </is>
       </c>
-      <c r="C16" s="20" t="n">
+      <c r="C16" s="21" t="n">
         <v>5000</v>
       </c>
-      <c r="D16" s="21" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E16" s="22" t="inlineStr">
+      <c r="E16" s="23" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="F16" s="21" t="inlineStr">
+      <c r="F16" s="22" t="inlineStr">
         <is>
           <t>Tech/software/ICT companies that hire engineers in-house.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Morocco</t>
         </is>
       </c>
-      <c r="C17" s="20" t="n">
+      <c r="C17" s="21" t="n">
         <v>2000</v>
       </c>
-      <c r="D17" s="21" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E17" s="22" t="inlineStr">
+      <c r="E17" s="23" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="F17" s="21" t="inlineStr">
+      <c r="F17" s="22" t="inlineStr">
         <is>
           <t>Tech/software/ICT companies that hire engineers in-house.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="14" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   KSA</t>
         </is>
       </c>
-      <c r="C18" s="20" t="n">
+      <c r="C18" s="21" t="n">
         <v>1800</v>
       </c>
-      <c r="D18" s="21" t="inlineStr">
+      <c r="D18" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E18" s="22" t="inlineStr">
+      <c r="E18" s="23" t="inlineStr">
         <is>
           <t>S5</t>
         </is>
       </c>
-      <c r="F18" s="21" t="inlineStr">
+      <c r="F18" s="22" t="inlineStr">
         <is>
           <t>Tech/software/ICT companies that hire engineers in-house.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Egypt</t>
         </is>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="21" t="n">
         <v>2500</v>
       </c>
-      <c r="D19" s="21" t="inlineStr">
+      <c r="D19" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E19" s="22" t="inlineStr">
+      <c r="E19" s="23" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="F19" s="21" t="inlineStr">
+      <c r="F19" s="22" t="inlineStr">
         <is>
           <t>Tech/software/ICT companies that hire engineers in-house.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>Mid-size firms w/ structured tech hiring (50-250)</t>
         </is>
       </c>
-      <c r="C20" s="19" t="n"/>
-      <c r="D20" s="19" t="n"/>
-      <c r="E20" s="19" t="n"/>
-      <c r="F20" s="19" t="n"/>
+      <c r="C20" s="20" t="n"/>
+      <c r="D20" s="20" t="n"/>
+      <c r="E20" s="20" t="n"/>
+      <c r="F20" s="20" t="n"/>
     </row>
     <row r="21">
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   France</t>
         </is>
       </c>
-      <c r="C21" s="20" t="n">
+      <c r="C21" s="21" t="n">
         <v>7300</v>
       </c>
-      <c r="D21" s="21" t="inlineStr">
+      <c r="D21" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E21" s="22" t="inlineStr">
+      <c r="E21" s="23" t="inlineStr">
         <is>
           <t>S1</t>
         </is>
       </c>
-      <c r="F21" s="21" t="inlineStr">
+      <c r="F21" s="22" t="inlineStr">
         <is>
           <t>Medium enterprises x share that run structured engineering hiring.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="B22" s="14" t="inlineStr">
+      <c r="B22" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   UK</t>
         </is>
       </c>
-      <c r="C22" s="20" t="n">
+      <c r="C22" s="21" t="n">
         <v>13200</v>
       </c>
-      <c r="D22" s="21" t="inlineStr">
+      <c r="D22" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E22" s="22" t="inlineStr">
+      <c r="E22" s="23" t="inlineStr">
         <is>
           <t>S2</t>
         </is>
       </c>
-      <c r="F22" s="21" t="inlineStr">
+      <c r="F22" s="22" t="inlineStr">
         <is>
           <t>Medium enterprises x share that run structured engineering hiring.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   UAE</t>
         </is>
       </c>
-      <c r="C23" s="20" t="n">
+      <c r="C23" s="21" t="n">
         <v>2800</v>
       </c>
-      <c r="D23" s="21" t="inlineStr">
+      <c r="D23" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E23" s="22" t="inlineStr">
+      <c r="E23" s="23" t="inlineStr">
         <is>
           <t>S3</t>
         </is>
       </c>
-      <c r="F23" s="21" t="inlineStr">
+      <c r="F23" s="22" t="inlineStr">
         <is>
           <t>Medium enterprises x share that run structured engineering hiring.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="14" t="inlineStr">
+      <c r="B24" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Morocco</t>
         </is>
       </c>
-      <c r="C24" s="20" t="n">
+      <c r="C24" s="21" t="n">
         <v>1250</v>
       </c>
-      <c r="D24" s="21" t="inlineStr">
+      <c r="D24" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E24" s="22" t="inlineStr">
+      <c r="E24" s="23" t="inlineStr">
         <is>
           <t>S4</t>
         </is>
       </c>
-      <c r="F24" s="21" t="inlineStr">
+      <c r="F24" s="22" t="inlineStr">
         <is>
           <t>Medium enterprises x share that run structured engineering hiring.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   KSA</t>
         </is>
       </c>
-      <c r="C25" s="20" t="n">
+      <c r="C25" s="21" t="n">
         <v>2600</v>
       </c>
-      <c r="D25" s="21" t="inlineStr">
+      <c r="D25" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E25" s="22" t="inlineStr">
+      <c r="E25" s="23" t="inlineStr">
         <is>
           <t>S5</t>
         </is>
       </c>
-      <c r="F25" s="21" t="inlineStr">
+      <c r="F25" s="22" t="inlineStr">
         <is>
           <t>Medium enterprises x share that run structured engineering hiring.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="14" t="inlineStr">
+      <c r="B26" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Egypt</t>
         </is>
       </c>
-      <c r="C26" s="20" t="n">
+      <c r="C26" s="21" t="n">
         <v>2000</v>
       </c>
-      <c r="D26" s="21" t="inlineStr">
+      <c r="D26" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E26" s="22" t="inlineStr">
+      <c r="E26" s="23" t="inlineStr">
         <is>
           <t>S6</t>
         </is>
       </c>
-      <c r="F26" s="21" t="inlineStr">
+      <c r="F26" s="22" t="inlineStr">
         <is>
           <t>Medium enterprises x share that run structured engineering hiring.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="18" t="inlineStr">
+      <c r="B27" s="19" t="inlineStr">
         <is>
           <t>Focus-6 subtotals (calc)</t>
         </is>
       </c>
-      <c r="C27" s="19" t="n"/>
-      <c r="D27" s="19" t="n"/>
-      <c r="E27" s="19" t="n"/>
-      <c r="F27" s="19" t="n"/>
+      <c r="C27" s="20" t="n"/>
+      <c r="D27" s="20" t="n"/>
+      <c r="E27" s="20" t="n"/>
+      <c r="F27" s="20" t="n"/>
     </row>
     <row r="28">
-      <c r="B28" s="14" t="inlineStr">
+      <c r="B28" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Agencies - focus-6 total</t>
         </is>
       </c>
-      <c r="C28" s="23">
+      <c r="C28" s="24">
         <f>(Assumptions!$C$7+Assumptions!$C$8+Assumptions!$C$9+Assumptions!$C$10+Assumptions!$C$11+Assumptions!$C$12)</f>
         <v/>
       </c>
-      <c r="D28" s="21" t="inlineStr">
+      <c r="D28" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E28" s="22" t="inlineStr"/>
-      <c r="F28" s="21" t="inlineStr">
+      <c r="E28" s="23" t="inlineStr"/>
+      <c r="F28" s="22" t="inlineStr">
         <is>
           <t>Sum across France, UK, UAE, Morocco, KSA, Egypt.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="B29" s="14" t="inlineStr">
+      <c r="B29" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Eng-heavy firms - focus-6 total</t>
         </is>
       </c>
-      <c r="C29" s="23">
+      <c r="C29" s="24">
         <f>(Assumptions!$C$14+Assumptions!$C$15+Assumptions!$C$16+Assumptions!$C$17+Assumptions!$C$18+Assumptions!$C$19)</f>
         <v/>
       </c>
-      <c r="D29" s="21" t="inlineStr">
+      <c r="D29" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E29" s="22" t="inlineStr"/>
-      <c r="F29" s="21" t="inlineStr">
+      <c r="E29" s="23" t="inlineStr"/>
+      <c r="F29" s="22" t="inlineStr">
         <is>
           <t>Sum across France, UK, UAE, Morocco, KSA, Egypt.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="14" t="inlineStr">
+      <c r="B30" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Mid-size firms - focus-6 total</t>
         </is>
       </c>
-      <c r="C30" s="23">
+      <c r="C30" s="24">
         <f>(Assumptions!$C$21+Assumptions!$C$22+Assumptions!$C$23+Assumptions!$C$24+Assumptions!$C$25+Assumptions!$C$26)</f>
         <v/>
       </c>
-      <c r="D30" s="21" t="inlineStr">
+      <c r="D30" s="22" t="inlineStr">
         <is>
           <t>entities</t>
         </is>
       </c>
-      <c r="E30" s="22" t="inlineStr"/>
-      <c r="F30" s="21" t="inlineStr">
+      <c r="E30" s="23" t="inlineStr"/>
+      <c r="F30" s="22" t="inlineStr">
         <is>
           <t>Sum across France, UK, UAE, Morocco, KSA, Egypt.</t>
         </is>
@@ -1476,63 +1516,63 @@
       <c r="F31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="B32" s="14" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>Agencies - % fit use case</t>
         </is>
       </c>
-      <c r="C32" s="24" t="n">
+      <c r="C32" s="25" t="n">
         <v>0.55</v>
       </c>
-      <c r="D32" s="21" t="inlineStr">
+      <c r="D32" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E32" s="22" t="inlineStr"/>
-      <c r="F32" s="21" t="inlineStr">
+      <c r="E32" s="23" t="inlineStr"/>
+      <c r="F32" s="22" t="inlineStr">
         <is>
           <t>Tech recruiting agencies run high req volume; structured assessment is core to their value-add. High fit.</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="15" t="inlineStr">
         <is>
           <t>Eng-heavy firms - % fit use case</t>
         </is>
       </c>
-      <c r="C33" s="24" t="n">
+      <c r="C33" s="25" t="n">
         <v>0.15</v>
       </c>
-      <c r="D33" s="21" t="inlineStr">
+      <c r="D33" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E33" s="22" t="inlineStr"/>
-      <c r="F33" s="21" t="inlineStr">
+      <c r="E33" s="23" t="inlineStr"/>
+      <c r="F33" s="22" t="inlineStr">
         <is>
           <t>Broad tech-firm base is ~95% micro (&lt;50 staff, solo dev shops). Only volume hirers run structured multi-candidate evaluation. Deliberately low.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B34" s="15" t="inlineStr">
         <is>
           <t>Mid-size firms - % fit use case</t>
         </is>
       </c>
-      <c r="C34" s="24" t="n">
+      <c r="C34" s="25" t="n">
         <v>0.25</v>
       </c>
-      <c r="D34" s="21" t="inlineStr">
+      <c r="D34" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E34" s="22" t="inlineStr"/>
-      <c r="F34" s="21" t="inlineStr">
+      <c r="E34" s="23" t="inlineStr"/>
+      <c r="F34" s="22" t="inlineStr">
         <is>
           <t>ICP pain (inconsistent evaluation) but lower adoption propensity / hire sporadically. Conservative.</t>
         </is>
@@ -1550,164 +1590,164 @@
       <c r="F35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B36" s="15" t="inlineStr">
         <is>
           <t>PAYG base price per test</t>
         </is>
       </c>
-      <c r="C36" s="25" t="n">
+      <c r="C36" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="D36" s="21" t="inlineStr">
+      <c r="D36" s="22" t="inlineStr">
         <is>
           <t>$/test</t>
         </is>
       </c>
-      <c r="E36" s="22" t="inlineStr">
+      <c r="E36" s="23" t="inlineStr">
         <is>
           <t>S7</t>
         </is>
       </c>
-      <c r="F36" s="21" t="inlineStr">
+      <c r="F36" s="22" t="inlineStr">
         <is>
           <t>Finalized BP base (was $15). Benchmark: TestGorilla ~$4.3/candidate, TestDome $7-20, HackerRank $15-20, Adaface entry $15. $14 sits at premium end.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="15" t="inlineStr">
         <is>
           <t>Small pack discount (20 tests)</t>
         </is>
       </c>
-      <c r="C37" s="26" t="n">
+      <c r="C37" s="27" t="n">
         <v>0.1</v>
       </c>
-      <c r="D37" s="21" t="inlineStr">
+      <c r="D37" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E37" s="22" t="inlineStr"/>
-      <c r="F37" s="21" t="inlineStr">
+      <c r="E37" s="23" t="inlineStr"/>
+      <c r="F37" s="22" t="inlineStr">
         <is>
           <t>Given.</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="14" t="inlineStr">
+      <c r="B38" s="15" t="inlineStr">
         <is>
           <t>Medium pack discount (100 tests)</t>
         </is>
       </c>
-      <c r="C38" s="26" t="n">
+      <c r="C38" s="27" t="n">
         <v>0.15</v>
       </c>
-      <c r="D38" s="21" t="inlineStr">
+      <c r="D38" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E38" s="22" t="inlineStr"/>
-      <c r="F38" s="21" t="inlineStr">
+      <c r="E38" s="23" t="inlineStr"/>
+      <c r="F38" s="22" t="inlineStr">
         <is>
           <t>Given.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="15" t="inlineStr">
         <is>
           <t>Enterprise pack discount (1,000 tests)</t>
         </is>
       </c>
-      <c r="C39" s="26" t="n">
+      <c r="C39" s="27" t="n">
         <v>0.2</v>
       </c>
-      <c r="D39" s="21" t="inlineStr">
+      <c r="D39" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E39" s="22" t="inlineStr"/>
-      <c r="F39" s="21" t="inlineStr">
+      <c r="E39" s="23" t="inlineStr"/>
+      <c r="F39" s="22" t="inlineStr">
         <is>
           <t>Finalized BP top tier: 1,000-test Enterprise pack at $11,200 (= $11.20/test). Replaces old 200-unit Large and the flat enterprise fee.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="14" t="inlineStr">
+      <c r="B40" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Net price - PAYG</t>
         </is>
       </c>
-      <c r="C40" s="27">
+      <c r="C40" s="28">
         <f>Assumptions!$C$36</f>
         <v/>
       </c>
-      <c r="D40" s="21" t="inlineStr">
+      <c r="D40" s="22" t="inlineStr">
         <is>
           <t>$/test</t>
         </is>
       </c>
-      <c r="E40" s="22" t="inlineStr"/>
-      <c r="F40" s="21" t="inlineStr"/>
+      <c r="E40" s="23" t="inlineStr"/>
+      <c r="F40" s="22" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="B41" s="14" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Net price - Small</t>
         </is>
       </c>
-      <c r="C41" s="27">
+      <c r="C41" s="28">
         <f>Assumptions!$C$36*(1-Assumptions!$C$37)</f>
         <v/>
       </c>
-      <c r="D41" s="21" t="inlineStr">
+      <c r="D41" s="22" t="inlineStr">
         <is>
           <t>$/test</t>
         </is>
       </c>
-      <c r="E41" s="22" t="inlineStr"/>
-      <c r="F41" s="21" t="inlineStr"/>
+      <c r="E41" s="23" t="inlineStr"/>
+      <c r="F41" s="22" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="B42" s="14" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Net price - Medium</t>
         </is>
       </c>
-      <c r="C42" s="27">
+      <c r="C42" s="28">
         <f>Assumptions!$C$36*(1-Assumptions!$C$38)</f>
         <v/>
       </c>
-      <c r="D42" s="21" t="inlineStr">
+      <c r="D42" s="22" t="inlineStr">
         <is>
           <t>$/test</t>
         </is>
       </c>
-      <c r="E42" s="22" t="inlineStr"/>
-      <c r="F42" s="21" t="inlineStr"/>
+      <c r="E42" s="23" t="inlineStr"/>
+      <c r="F42" s="22" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="B43" s="14" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Net price - Enterprise (1,000-pack)</t>
         </is>
       </c>
-      <c r="C43" s="27">
+      <c r="C43" s="28">
         <f>Assumptions!$C$36*(1-Assumptions!$C$39)</f>
         <v/>
       </c>
-      <c r="D43" s="21" t="inlineStr">
+      <c r="D43" s="22" t="inlineStr">
         <is>
           <t>$/test</t>
         </is>
       </c>
-      <c r="E43" s="22" t="inlineStr"/>
-      <c r="F43" s="21" t="inlineStr"/>
+      <c r="E43" s="23" t="inlineStr"/>
+      <c r="F43" s="22" t="inlineStr"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="B44" s="4" t="inlineStr">
@@ -1721,120 +1761,120 @@
       <c r="F44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="B45" s="14" t="inlineStr">
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>PAYG share</t>
         </is>
       </c>
-      <c r="C45" s="26" t="n">
+      <c r="C45" s="27" t="n">
         <v>0.1</v>
       </c>
-      <c r="D45" s="21" t="inlineStr">
+      <c r="D45" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E45" s="22" t="inlineStr"/>
-      <c r="F45" s="21" t="inlineStr">
+      <c r="E45" s="23" t="inlineStr"/>
+      <c r="F45" s="22" t="inlineStr">
         <is>
           <t>Finalized BP is pack-led; PAYG is a thin trial tier, not the base.</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="B46" s="14" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>Small pack share</t>
         </is>
       </c>
-      <c r="C46" s="26" t="n">
+      <c r="C46" s="27" t="n">
         <v>0.35</v>
       </c>
-      <c r="D46" s="21" t="inlineStr">
+      <c r="D46" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E46" s="22" t="inlineStr"/>
-      <c r="F46" s="21" t="inlineStr"/>
+      <c r="E46" s="23" t="inlineStr"/>
+      <c r="F46" s="22" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="B47" s="14" t="inlineStr">
+      <c r="B47" s="15" t="inlineStr">
         <is>
           <t>Medium pack share</t>
         </is>
       </c>
-      <c r="C47" s="26" t="n">
+      <c r="C47" s="27" t="n">
         <v>0.35</v>
       </c>
-      <c r="D47" s="21" t="inlineStr">
+      <c r="D47" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E47" s="22" t="inlineStr"/>
-      <c r="F47" s="21" t="inlineStr"/>
+      <c r="E47" s="23" t="inlineStr"/>
+      <c r="F47" s="22" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="B48" s="14" t="inlineStr">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>Enterprise (1,000-pack) share</t>
         </is>
       </c>
-      <c r="C48" s="26" t="n">
+      <c r="C48" s="27" t="n">
         <v>0.2</v>
       </c>
-      <c r="D48" s="21" t="inlineStr">
+      <c r="D48" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E48" s="22" t="inlineStr"/>
-      <c r="F48" s="21" t="inlineStr">
+      <c r="E48" s="23" t="inlineStr"/>
+      <c r="F48" s="22" t="inlineStr">
         <is>
           <t>Heaviest buyers; matches finalized BP customer mix.</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="B49" s="14" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Mix check (=100%)</t>
         </is>
       </c>
-      <c r="C49" s="28">
+      <c r="C49" s="29">
         <f>Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48</f>
         <v/>
       </c>
-      <c r="D49" s="21" t="inlineStr">
+      <c r="D49" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E49" s="22" t="inlineStr"/>
-      <c r="F49" s="21" t="inlineStr">
+      <c r="E49" s="23" t="inlineStr"/>
+      <c r="F49" s="22" t="inlineStr">
         <is>
           <t>Must equal 100%.</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="B50" s="14" t="inlineStr">
+      <c r="B50" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Blended net price per test</t>
         </is>
       </c>
-      <c r="C50" s="27">
+      <c r="C50" s="28">
         <f>(Assumptions!$C$45*Assumptions!$C$40+Assumptions!$C$46*Assumptions!$C$41+Assumptions!$C$47*Assumptions!$C$42+Assumptions!$C$48*Assumptions!$C$43)/(Assumptions!$C$45+Assumptions!$C$46+Assumptions!$C$47+Assumptions!$C$48)</f>
         <v/>
       </c>
-      <c r="D50" s="21" t="inlineStr">
+      <c r="D50" s="22" t="inlineStr">
         <is>
           <t>$/test</t>
         </is>
       </c>
-      <c r="E50" s="22" t="inlineStr"/>
-      <c r="F50" s="21" t="inlineStr">
+      <c r="E50" s="23" t="inlineStr"/>
+      <c r="F50" s="22" t="inlineStr">
         <is>
           <t>Mix-weighted net price across all four packs.</t>
         </is>
@@ -1852,261 +1892,261 @@
       <c r="F51" s="5" t="n"/>
     </row>
     <row r="52">
-      <c r="B52" s="14" t="inlineStr">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>Tests-per-account scalar (sensitivity handle)</t>
         </is>
       </c>
-      <c r="C52" s="29" t="n">
+      <c r="C52" s="30" t="n">
         <v>1</v>
       </c>
-      <c r="D52" s="21" t="inlineStr">
+      <c r="D52" s="22" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="E52" s="22" t="inlineStr"/>
-      <c r="F52" s="21" t="inlineStr">
+      <c r="E52" s="23" t="inlineStr"/>
+      <c r="F52" s="22" t="inlineStr">
         <is>
           <t>Global multiplier on tests/account. Base=1.00; flex in sensitivity.</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="B53" s="14" t="inlineStr">
+      <c r="B53" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Agencies - roles hired / yr</t>
         </is>
       </c>
-      <c r="C53" s="20" t="n">
+      <c r="C53" s="21" t="n">
         <v>80</v>
       </c>
-      <c r="D53" s="21" t="inlineStr">
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>roles</t>
         </is>
       </c>
-      <c r="E53" s="22" t="inlineStr"/>
-      <c r="F53" s="21" t="inlineStr">
+      <c r="E53" s="23" t="inlineStr"/>
+      <c r="F53" s="22" t="inlineStr">
         <is>
           <t>High req throughput - many client roles, several candidates screened each.</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="B54" s="14" t="inlineStr">
+      <c r="B54" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Agencies - candidates tested / role</t>
         </is>
       </c>
-      <c r="C54" s="20" t="n">
+      <c r="C54" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="D54" s="21" t="inlineStr">
+      <c r="D54" s="22" t="inlineStr">
         <is>
           <t>cand</t>
         </is>
       </c>
-      <c r="E54" s="22" t="inlineStr"/>
-      <c r="F54" s="21" t="inlineStr"/>
+      <c r="E54" s="23" t="inlineStr"/>
+      <c r="F54" s="22" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="B55" s="14" t="inlineStr">
+      <c r="B55" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Agencies - tests / account / yr</t>
         </is>
       </c>
-      <c r="C55" s="23">
+      <c r="C55" s="24">
         <f>Assumptions!$C$53*Assumptions!$C$54*Assumptions!$C$52</f>
         <v/>
       </c>
-      <c r="D55" s="21" t="inlineStr">
+      <c r="D55" s="22" t="inlineStr">
         <is>
           <t>tests</t>
         </is>
       </c>
-      <c r="E55" s="22" t="inlineStr"/>
-      <c r="F55" s="21" t="inlineStr">
+      <c r="E55" s="23" t="inlineStr"/>
+      <c r="F55" s="22" t="inlineStr">
         <is>
           <t>roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="B56" s="14" t="inlineStr">
+      <c r="B56" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Eng-heavy firms - roles hired / yr</t>
         </is>
       </c>
-      <c r="C56" s="20" t="n">
+      <c r="C56" s="21" t="n">
         <v>25</v>
       </c>
-      <c r="D56" s="21" t="inlineStr">
+      <c r="D56" s="22" t="inlineStr">
         <is>
           <t>roles</t>
         </is>
       </c>
-      <c r="E56" s="22" t="inlineStr"/>
-      <c r="F56" s="21" t="inlineStr">
+      <c r="E56" s="23" t="inlineStr"/>
+      <c r="F56" s="22" t="inlineStr">
         <is>
           <t>Steady in-house eng hiring.</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="B57" s="14" t="inlineStr">
+      <c r="B57" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Eng-heavy firms - candidates tested / role</t>
         </is>
       </c>
-      <c r="C57" s="20" t="n">
+      <c r="C57" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="D57" s="21" t="inlineStr">
+      <c r="D57" s="22" t="inlineStr">
         <is>
           <t>cand</t>
         </is>
       </c>
-      <c r="E57" s="22" t="inlineStr"/>
-      <c r="F57" s="21" t="inlineStr"/>
+      <c r="E57" s="23" t="inlineStr"/>
+      <c r="F57" s="22" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="B58" s="14" t="inlineStr">
+      <c r="B58" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Eng-heavy firms - tests / account / yr</t>
         </is>
       </c>
-      <c r="C58" s="23">
+      <c r="C58" s="24">
         <f>Assumptions!$C$56*Assumptions!$C$57*Assumptions!$C$52</f>
         <v/>
       </c>
-      <c r="D58" s="21" t="inlineStr">
+      <c r="D58" s="22" t="inlineStr">
         <is>
           <t>tests</t>
         </is>
       </c>
-      <c r="E58" s="22" t="inlineStr"/>
-      <c r="F58" s="21" t="inlineStr">
+      <c r="E58" s="23" t="inlineStr"/>
+      <c r="F58" s="22" t="inlineStr">
         <is>
           <t>roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="B59" s="14" t="inlineStr">
+      <c r="B59" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Mid-size firms - roles hired / yr</t>
         </is>
       </c>
-      <c r="C59" s="20" t="n">
+      <c r="C59" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="D59" s="21" t="inlineStr">
+      <c r="D59" s="22" t="inlineStr">
         <is>
           <t>roles</t>
         </is>
       </c>
-      <c r="E59" s="22" t="inlineStr"/>
-      <c r="F59" s="21" t="inlineStr">
+      <c r="E59" s="23" t="inlineStr"/>
+      <c r="F59" s="22" t="inlineStr">
         <is>
           <t>Sporadic, lower-volume hiring.</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="B60" s="14" t="inlineStr">
+      <c r="B60" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Mid-size firms - candidates tested / role</t>
         </is>
       </c>
-      <c r="C60" s="20" t="n">
+      <c r="C60" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="D60" s="21" t="inlineStr">
+      <c r="D60" s="22" t="inlineStr">
         <is>
           <t>cand</t>
         </is>
       </c>
-      <c r="E60" s="22" t="inlineStr"/>
-      <c r="F60" s="21" t="inlineStr"/>
+      <c r="E60" s="23" t="inlineStr"/>
+      <c r="F60" s="22" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="B61" s="14" t="inlineStr">
+      <c r="B61" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Mid-size firms - tests / account / yr</t>
         </is>
       </c>
-      <c r="C61" s="23">
+      <c r="C61" s="24">
         <f>Assumptions!$C$59*Assumptions!$C$60*Assumptions!$C$52</f>
         <v/>
       </c>
-      <c r="D61" s="21" t="inlineStr">
+      <c r="D61" s="22" t="inlineStr">
         <is>
           <t>tests</t>
         </is>
       </c>
-      <c r="E61" s="22" t="inlineStr"/>
-      <c r="F61" s="21" t="inlineStr">
+      <c r="E61" s="23" t="inlineStr"/>
+      <c r="F61" s="22" t="inlineStr">
         <is>
           <t>roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="B62" s="14" t="inlineStr">
+      <c r="B62" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Channel acct - roles hired / yr</t>
         </is>
       </c>
-      <c r="C62" s="20" t="n">
+      <c r="C62" s="21" t="n">
         <v>40</v>
       </c>
-      <c r="D62" s="21" t="inlineStr">
+      <c r="D62" s="22" t="inlineStr">
         <is>
           <t>roles</t>
         </is>
       </c>
-      <c r="E62" s="22" t="inlineStr"/>
-      <c r="F62" s="21" t="inlineStr">
+      <c r="E62" s="23" t="inlineStr"/>
+      <c r="F62" s="22" t="inlineStr">
         <is>
           <t>Manatal users: mix of agencies + in-house recruiters.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="B63" s="14" t="inlineStr">
+      <c r="B63" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Channel acct - candidates tested / role</t>
         </is>
       </c>
-      <c r="C63" s="20" t="n">
+      <c r="C63" s="21" t="n">
         <v>5</v>
       </c>
-      <c r="D63" s="21" t="inlineStr">
+      <c r="D63" s="22" t="inlineStr">
         <is>
           <t>cand</t>
         </is>
       </c>
-      <c r="E63" s="22" t="inlineStr"/>
-      <c r="F63" s="21" t="inlineStr"/>
+      <c r="E63" s="23" t="inlineStr"/>
+      <c r="F63" s="22" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="B64" s="14" t="inlineStr">
+      <c r="B64" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Channel acct - tests / account / yr</t>
         </is>
       </c>
-      <c r="C64" s="23">
+      <c r="C64" s="24">
         <f>Assumptions!$C$62*Assumptions!$C$63*Assumptions!$C$52</f>
         <v/>
       </c>
-      <c r="D64" s="21" t="inlineStr">
+      <c r="D64" s="22" t="inlineStr">
         <is>
           <t>tests</t>
         </is>
       </c>
-      <c r="E64" s="22" t="inlineStr"/>
-      <c r="F64" s="21" t="inlineStr"/>
+      <c r="E64" s="23" t="inlineStr"/>
+      <c r="F64" s="22" t="inlineStr"/>
     </row>
     <row r="65" ht="20" customHeight="1">
       <c r="B65" s="4" t="inlineStr">
@@ -2120,88 +2160,88 @@
       <c r="F65" s="5" t="n"/>
     </row>
     <row r="66">
-      <c r="B66" s="14" t="inlineStr">
+      <c r="B66" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Agencies - ACV / account / yr</t>
         </is>
       </c>
-      <c r="C66" s="23">
+      <c r="C66" s="24">
         <f>Assumptions!$C$55*Assumptions!$C$50</f>
         <v/>
       </c>
-      <c r="D66" s="21" t="inlineStr">
+      <c r="D66" s="22" t="inlineStr">
         <is>
           <t>$/yr</t>
         </is>
       </c>
-      <c r="E66" s="22" t="inlineStr"/>
-      <c r="F66" s="21" t="inlineStr">
+      <c r="E66" s="23" t="inlineStr"/>
+      <c r="F66" s="22" t="inlineStr">
         <is>
           <t>tests/account x blended net price per test.</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="B67" s="14" t="inlineStr">
+      <c r="B67" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Eng-heavy firms - ACV / account / yr</t>
         </is>
       </c>
-      <c r="C67" s="23">
+      <c r="C67" s="24">
         <f>Assumptions!$C$58*Assumptions!$C$50</f>
         <v/>
       </c>
-      <c r="D67" s="21" t="inlineStr">
+      <c r="D67" s="22" t="inlineStr">
         <is>
           <t>$/yr</t>
         </is>
       </c>
-      <c r="E67" s="22" t="inlineStr"/>
-      <c r="F67" s="21" t="inlineStr">
+      <c r="E67" s="23" t="inlineStr"/>
+      <c r="F67" s="22" t="inlineStr">
         <is>
           <t>tests/account x blended net price per test.</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="B68" s="14" t="inlineStr">
+      <c r="B68" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Mid-size firms - ACV / account / yr</t>
         </is>
       </c>
-      <c r="C68" s="23">
+      <c r="C68" s="24">
         <f>Assumptions!$C$61*Assumptions!$C$50</f>
         <v/>
       </c>
-      <c r="D68" s="21" t="inlineStr">
+      <c r="D68" s="22" t="inlineStr">
         <is>
           <t>$/yr</t>
         </is>
       </c>
-      <c r="E68" s="22" t="inlineStr"/>
-      <c r="F68" s="21" t="inlineStr">
+      <c r="E68" s="23" t="inlineStr"/>
+      <c r="F68" s="22" t="inlineStr">
         <is>
           <t>tests/account x blended net price per test.</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="B69" s="14" t="inlineStr">
+      <c r="B69" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">   Channel acct - ACV / account / yr</t>
         </is>
       </c>
-      <c r="C69" s="23">
+      <c r="C69" s="24">
         <f>Assumptions!$C$64*Assumptions!$C$50</f>
         <v/>
       </c>
-      <c r="D69" s="21" t="inlineStr">
+      <c r="D69" s="22" t="inlineStr">
         <is>
           <t>$/yr</t>
         </is>
       </c>
-      <c r="E69" s="22" t="inlineStr"/>
-      <c r="F69" s="21" t="inlineStr">
+      <c r="E69" s="23" t="inlineStr"/>
+      <c r="F69" s="22" t="inlineStr">
         <is>
           <t>tests/account x blended net price per test.</t>
         </is>
@@ -2219,155 +2259,155 @@
       <c r="F70" s="5" t="n"/>
     </row>
     <row r="71">
-      <c r="B71" s="14" t="inlineStr">
+      <c r="B71" s="15" t="inlineStr">
         <is>
           <t>Manatal client base</t>
         </is>
       </c>
-      <c r="C71" s="20" t="n">
+      <c r="C71" s="21" t="n">
         <v>10000</v>
       </c>
-      <c r="D71" s="21" t="inlineStr">
+      <c r="D71" s="22" t="inlineStr">
         <is>
           <t>clients</t>
         </is>
       </c>
-      <c r="E71" s="22" t="inlineStr">
+      <c r="E71" s="23" t="inlineStr">
         <is>
           <t>S8</t>
         </is>
       </c>
-      <c r="F71" s="21" t="inlineStr">
+      <c r="F71" s="22" t="inlineStr">
         <is>
           <t>Anchor: embedded in Manatal, 10,000+ clients / 100+ countries.</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="B72" s="14" t="inlineStr">
+      <c r="B72" s="15" t="inlineStr">
         <is>
           <t>ICP-relevant share of Manatal base</t>
         </is>
       </c>
-      <c r="C72" s="26" t="n">
+      <c r="C72" s="27" t="n">
         <v>0.45</v>
       </c>
-      <c r="D72" s="21" t="inlineStr">
+      <c r="D72" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E72" s="22" t="inlineStr"/>
-      <c r="F72" s="21" t="inlineStr">
+      <c r="E72" s="23" t="inlineStr"/>
+      <c r="F72" s="22" t="inlineStr">
         <is>
           <t>Manatal is a recruiter/agency ATS - most clients actively hire for roles Invirtus can assess.</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="B73" s="14" t="inlineStr">
+      <c r="B73" s="15" t="inlineStr">
         <is>
           <t>Attach rate - year 1</t>
         </is>
       </c>
-      <c r="C73" s="24" t="n">
+      <c r="C73" s="25" t="n">
         <v>0.02</v>
       </c>
-      <c r="D73" s="21" t="inlineStr">
+      <c r="D73" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E73" s="22" t="inlineStr"/>
-      <c r="F73" s="21" t="inlineStr">
+      <c r="E73" s="23" t="inlineStr"/>
+      <c r="F73" s="22" t="inlineStr">
         <is>
           <t>Share of relevant Manatal clients activating Invirtus. Embedded distribution, low early activation.</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="B74" s="14" t="inlineStr">
+      <c r="B74" s="15" t="inlineStr">
         <is>
           <t>Attach rate - year 2</t>
         </is>
       </c>
-      <c r="C74" s="24" t="n">
+      <c r="C74" s="25" t="n">
         <v>0.05</v>
       </c>
-      <c r="D74" s="21" t="inlineStr">
+      <c r="D74" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E74" s="22" t="inlineStr"/>
-      <c r="F74" s="21" t="inlineStr">
+      <c r="E74" s="23" t="inlineStr"/>
+      <c r="F74" s="22" t="inlineStr">
         <is>
           <t>Ramp.</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="B75" s="14" t="inlineStr">
+      <c r="B75" s="15" t="inlineStr">
         <is>
           <t>Attach rate - year 3 (SOM)</t>
         </is>
       </c>
-      <c r="C75" s="24" t="n">
+      <c r="C75" s="25" t="n">
         <v>0.08</v>
       </c>
-      <c r="D75" s="21" t="inlineStr">
+      <c r="D75" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E75" s="22" t="inlineStr"/>
-      <c r="F75" s="21" t="inlineStr">
+      <c r="E75" s="23" t="inlineStr"/>
+      <c r="F75" s="22" t="inlineStr">
         <is>
           <t>BIGGEST SOM DRIVER. Realistic embedded-tool attach, not best-in-class.</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="B76" s="14" t="inlineStr">
+      <c r="B76" s="15" t="inlineStr">
         <is>
           <t>Include 2nd ATS (Socium) in base?  (1/0)</t>
         </is>
       </c>
-      <c r="C76" s="30" t="n">
+      <c r="C76" s="31" t="n">
         <v>0</v>
       </c>
-      <c r="D76" s="21" t="inlineStr">
+      <c r="D76" s="22" t="inlineStr">
         <is>
           <t>flag</t>
         </is>
       </c>
-      <c r="E76" s="22" t="inlineStr"/>
-      <c r="F76" s="21" t="inlineStr">
+      <c r="E76" s="23" t="inlineStr"/>
+      <c r="F76" s="22" t="inlineStr">
         <is>
           <t>Held as UPSIDE until integration is real. Set 1 to include.</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="B77" s="14" t="inlineStr">
+      <c r="B77" s="15" t="inlineStr">
         <is>
           <t>Socium client base (upside)</t>
         </is>
       </c>
-      <c r="C77" s="20" t="n">
+      <c r="C77" s="21" t="n">
         <v>3000</v>
       </c>
-      <c r="D77" s="21" t="inlineStr">
+      <c r="D77" s="22" t="inlineStr">
         <is>
           <t>clients</t>
         </is>
       </c>
-      <c r="E77" s="22" t="inlineStr">
+      <c r="E77" s="23" t="inlineStr">
         <is>
           <t>S9</t>
         </is>
       </c>
-      <c r="F77" s="21" t="inlineStr">
+      <c r="F77" s="22" t="inlineStr">
         <is>
           <t>Upside only.</t>
         </is>
@@ -2385,84 +2425,84 @@
       <c r="F78" s="5" t="n"/>
     </row>
     <row r="79">
-      <c r="B79" s="14" t="inlineStr">
+      <c r="B79" s="15" t="inlineStr">
         <is>
           <t>3-yr penetration of serviceable SAM accounts</t>
         </is>
       </c>
-      <c r="C79" s="24" t="n">
+      <c r="C79" s="25" t="n">
         <v>0.008</v>
       </c>
-      <c r="D79" s="21" t="inlineStr">
+      <c r="D79" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E79" s="22" t="inlineStr"/>
-      <c r="F79" s="21" t="inlineStr">
+      <c r="E79" s="23" t="inlineStr"/>
+      <c r="F79" s="22" t="inlineStr">
         <is>
           <t>Direct capture is gated by low trial-to-paid; a pre-seed wins only a thin slice of the large serviceable base.</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="B80" s="14" t="inlineStr">
+      <c r="B80" s="15" t="inlineStr">
         <is>
           <t>Monthly website traffic</t>
         </is>
       </c>
-      <c r="C80" s="20" t="n">
+      <c r="C80" s="21" t="n">
         <v>8000</v>
       </c>
-      <c r="D80" s="21" t="inlineStr">
+      <c r="D80" s="22" t="inlineStr">
         <is>
           <t>visits/mo</t>
         </is>
       </c>
-      <c r="E80" s="22" t="inlineStr"/>
-      <c r="F80" s="21" t="inlineStr">
+      <c r="E80" s="23" t="inlineStr"/>
+      <c r="F80" s="22" t="inlineStr">
         <is>
           <t>Self-serve funnel cross-check input (year-3 run-rate).</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="B81" s="14" t="inlineStr">
+      <c r="B81" s="15" t="inlineStr">
         <is>
           <t>Visit -&gt; free-trial conversion</t>
         </is>
       </c>
-      <c r="C81" s="24" t="n">
+      <c r="C81" s="25" t="n">
         <v>0.03</v>
       </c>
-      <c r="D81" s="21" t="inlineStr">
+      <c r="D81" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E81" s="22" t="inlineStr"/>
-      <c r="F81" s="21" t="inlineStr"/>
+      <c r="E81" s="23" t="inlineStr"/>
+      <c r="F81" s="22" t="inlineStr"/>
     </row>
     <row r="82">
-      <c r="B82" s="14" t="inlineStr">
+      <c r="B82" s="15" t="inlineStr">
         <is>
           <t>Trial -&gt; paid conversion</t>
         </is>
       </c>
-      <c r="C82" s="24" t="n">
+      <c r="C82" s="25" t="n">
         <v>0.05</v>
       </c>
-      <c r="D82" s="21" t="inlineStr">
+      <c r="D82" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E82" s="22" t="inlineStr">
+      <c r="E82" s="23" t="inlineStr">
         <is>
           <t>S8</t>
         </is>
       </c>
-      <c r="F82" s="21" t="inlineStr">
+      <c r="F82" s="22" t="inlineStr">
         <is>
           <t>Currently LOW - do NOT assume best-in-class. Flagged in GTM notes.</t>
         </is>
@@ -2480,46 +2520,46 @@
       <c r="F83" s="5" t="n"/>
     </row>
     <row r="84">
-      <c r="B84" s="14" t="inlineStr">
+      <c r="B84" s="15" t="inlineStr">
         <is>
           <t>Steady-state annual retention</t>
         </is>
       </c>
-      <c r="C84" s="24" t="n">
+      <c r="C84" s="25" t="n">
         <v>0.9</v>
       </c>
-      <c r="D84" s="21" t="inlineStr">
+      <c r="D84" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E84" s="22" t="inlineStr">
+      <c r="E84" s="23" t="inlineStr">
         <is>
           <t>S8</t>
         </is>
       </c>
-      <c r="F84" s="21" t="inlineStr">
+      <c r="F84" s="22" t="inlineStr">
         <is>
           <t>Finalized BP assumes 7% gross churn (93% retention); held slightly conservative at 90% for the SOM. 100% to date on a tiny base.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="B85" s="14" t="inlineStr">
+      <c r="B85" s="15" t="inlineStr">
         <is>
           <t>Focus-6 share of global addressable universe</t>
         </is>
       </c>
-      <c r="C85" s="24" t="n">
+      <c r="C85" s="25" t="n">
         <v>0.12</v>
       </c>
-      <c r="D85" s="21" t="inlineStr">
+      <c r="D85" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E85" s="22" t="inlineStr"/>
-      <c r="F85" s="21" t="inlineStr">
+      <c r="E85" s="23" t="inlineStr"/>
+      <c r="F85" s="22" t="inlineStr">
         <is>
           <t>Focus-6 as % of all geos where product works. Grosses SAM up to TAM. US/India/rest-EU dominate.</t>
         </is>
@@ -2537,69 +2577,130 @@
       <c r="F86" s="5" t="n"/>
     </row>
     <row r="87">
-      <c r="B87" s="14" t="inlineStr">
+      <c r="B87" s="15" t="inlineStr">
         <is>
           <t>Cost of a bad hire</t>
         </is>
       </c>
-      <c r="C87" s="20" t="n">
+      <c r="C87" s="21" t="n">
         <v>150000</v>
       </c>
-      <c r="D87" s="21" t="inlineStr">
+      <c r="D87" s="22" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="E87" s="22" t="inlineStr">
+      <c r="E87" s="23" t="inlineStr">
         <is>
           <t>S8</t>
         </is>
       </c>
-      <c r="F87" s="21" t="inlineStr">
+      <c r="F87" s="22" t="inlineStr">
         <is>
           <t>Core value anchor used across sales &amp; fundraising.</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="B88" s="14" t="inlineStr">
+      <c r="B88" s="15" t="inlineStr">
         <is>
           <t>Tests run per hire placed</t>
         </is>
       </c>
-      <c r="C88" s="20" t="n">
+      <c r="C88" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="D88" s="21" t="inlineStr">
+      <c r="D88" s="22" t="inlineStr">
         <is>
           <t>tests</t>
         </is>
       </c>
-      <c r="E88" s="22" t="inlineStr"/>
-      <c r="F88" s="21" t="inlineStr">
+      <c r="E88" s="23" t="inlineStr"/>
+      <c r="F88" s="22" t="inlineStr">
         <is>
           <t>Candidates assessed per filled role (1 hire/role).</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="B89" s="14" t="inlineStr">
+      <c r="B89" s="15" t="inlineStr">
         <is>
           <t>Bad-hire rate reduction from structured eval</t>
         </is>
       </c>
-      <c r="C89" s="26" t="n">
+      <c r="C89" s="27" t="n">
         <v>0.2</v>
       </c>
-      <c r="D89" s="21" t="inlineStr">
+      <c r="D89" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="E89" s="22" t="inlineStr"/>
-      <c r="F89" s="21" t="inlineStr">
+      <c r="E89" s="23" t="inlineStr"/>
+      <c r="F89" s="22" t="inlineStr">
         <is>
           <t>Assumed share of bad-hire cost avoided via better screening.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="20" customHeight="1">
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>11. Talent-DB monetization  (2nd revenue stream)  [finalized BP]</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="n"/>
+      <c r="D90" s="5" t="n"/>
+      <c r="E90" s="5" t="n"/>
+      <c r="F90" s="5" t="n"/>
+    </row>
+    <row r="91">
+      <c r="B91" s="15" t="inlineStr">
+        <is>
+          <t>Profiles sourced from own DB (mature)</t>
+        </is>
+      </c>
+      <c r="C91" s="25" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D91" s="22" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="E91" s="23" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="F91" s="22" t="inlineStr">
+        <is>
+          <t>Finalized BP ramps 1% (2026) -&gt; 50% (2030); 30% used as mature steady-state. Profiles sourced = tests run x this %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="15" t="inlineStr">
+        <is>
+          <t>Avg price per sourced profile</t>
+        </is>
+      </c>
+      <c r="C92" s="21" t="n">
+        <v>30</v>
+      </c>
+      <c r="D92" s="22" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="E92" s="23" t="inlineStr">
+        <is>
+          <t>S7</t>
+        </is>
+      </c>
+      <c r="F92" s="22" t="inlineStr">
+        <is>
+          <t>Finalized BP: $30 per sourced profile, flat.</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2718,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:H40"/>
+  <dimension ref="B1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2631,16 +2732,16 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="16" t="inlineStr">
-        <is>
-          <t>INVIRTUS  -  TAM / SAM / SOM build</t>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>INVIRTUS  -  Revenue potential build  (TAM / SAM / SOM)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="17" t="inlineStr">
-        <is>
-          <t>Bottoms-up: entities x %fit x tests/yr x net $/test. USD. All drivers live on Assumptions.</t>
+      <c r="B2" s="18" t="inlineStr">
+        <is>
+          <t>Bottoms-up: entities x %fit x tests/yr x net $/test, plus talent-DB stream. USD. All drivers live on Assumptions.</t>
         </is>
       </c>
     </row>
@@ -2658,37 +2759,37 @@
       <c r="H4" s="5" t="n"/>
     </row>
     <row r="5">
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="32" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="32" t="inlineStr">
         <is>
           <t>Entities (focus-6)</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="D5" s="32" t="inlineStr">
         <is>
           <t>% fit</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="32" t="inlineStr">
         <is>
           <t>Serviceable accts</t>
         </is>
       </c>
-      <c r="F5" s="31" t="inlineStr">
+      <c r="F5" s="32" t="inlineStr">
         <is>
           <t>Tests/acct/yr</t>
         </is>
       </c>
-      <c r="G5" s="31" t="inlineStr">
+      <c r="G5" s="32" t="inlineStr">
         <is>
           <t>ACV/acct ($)</t>
         </is>
       </c>
-      <c r="H5" s="31" t="inlineStr">
+      <c r="H5" s="32" t="inlineStr">
         <is>
           <t>SAM value ($/yr)</t>
         </is>
@@ -2700,27 +2801,27 @@
           <t>Tech recruiting agencies</t>
         </is>
       </c>
-      <c r="C6" s="32">
+      <c r="C6" s="33">
         <f>Assumptions!$C$28</f>
         <v/>
       </c>
-      <c r="D6" s="33">
+      <c r="D6" s="34">
         <f>Assumptions!$C$32</f>
         <v/>
       </c>
-      <c r="E6" s="32">
+      <c r="E6" s="33">
         <f>C6*D6</f>
         <v/>
       </c>
-      <c r="F6" s="32">
+      <c r="F6" s="33">
         <f>Assumptions!$C$55</f>
         <v/>
       </c>
-      <c r="G6" s="32">
+      <c r="G6" s="33">
         <f>Assumptions!$C$66</f>
         <v/>
       </c>
-      <c r="H6" s="32">
+      <c r="H6" s="33">
         <f>E6*G6</f>
         <v/>
       </c>
@@ -2731,27 +2832,27 @@
           <t>Engineering-heavy firms</t>
         </is>
       </c>
-      <c r="C7" s="32">
+      <c r="C7" s="33">
         <f>Assumptions!$C$29</f>
         <v/>
       </c>
-      <c r="D7" s="33">
+      <c r="D7" s="34">
         <f>Assumptions!$C$33</f>
         <v/>
       </c>
-      <c r="E7" s="32">
+      <c r="E7" s="33">
         <f>C7*D7</f>
         <v/>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="33">
         <f>Assumptions!$C$58</f>
         <v/>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="33">
         <f>Assumptions!$C$67</f>
         <v/>
       </c>
-      <c r="H7" s="32">
+      <c r="H7" s="33">
         <f>E7*G7</f>
         <v/>
       </c>
@@ -2762,33 +2863,33 @@
           <t>Mid-size structured-hiring firms</t>
         </is>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="33">
         <f>Assumptions!$C$30</f>
         <v/>
       </c>
-      <c r="D8" s="33">
+      <c r="D8" s="34">
         <f>Assumptions!$C$34</f>
         <v/>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="33">
         <f>C8*D8</f>
         <v/>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="33">
         <f>Assumptions!$C$61</f>
         <v/>
       </c>
-      <c r="G8" s="32">
+      <c r="G8" s="33">
         <f>Assumptions!$C$68</f>
         <v/>
       </c>
-      <c r="H8" s="32">
+      <c r="H8" s="33">
         <f>E8*G8</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="34" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>SAM  (focus-6, serviceable today)</t>
         </is>
@@ -2823,32 +2924,32 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="31" t="inlineStr">
+      <c r="B13" s="32" t="inlineStr">
         <is>
           <t>Segment</t>
         </is>
       </c>
-      <c r="C13" s="31" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>Global entities</t>
         </is>
       </c>
-      <c r="D13" s="31" t="inlineStr">
+      <c r="D13" s="32" t="inlineStr">
         <is>
           <t>% fit</t>
         </is>
       </c>
-      <c r="E13" s="31" t="inlineStr">
+      <c r="E13" s="32" t="inlineStr">
         <is>
           <t>Serviceable accts</t>
         </is>
       </c>
-      <c r="F13" s="31" t="inlineStr">
+      <c r="F13" s="32" t="inlineStr">
         <is>
           <t>ACV/acct ($)</t>
         </is>
       </c>
-      <c r="G13" s="31" t="inlineStr">
+      <c r="G13" s="32" t="inlineStr">
         <is>
           <t>TAM value ($/yr)</t>
         </is>
@@ -2860,23 +2961,23 @@
           <t>Tech recruiting agencies</t>
         </is>
       </c>
-      <c r="C14" s="32">
+      <c r="C14" s="33">
         <f>Assumptions!$C$28/Assumptions!$C$85</f>
         <v/>
       </c>
-      <c r="D14" s="33">
+      <c r="D14" s="34">
         <f>Assumptions!$C$32</f>
         <v/>
       </c>
-      <c r="E14" s="32">
+      <c r="E14" s="33">
         <f>C14*D14</f>
         <v/>
       </c>
-      <c r="F14" s="32">
+      <c r="F14" s="33">
         <f>Assumptions!$C$66</f>
         <v/>
       </c>
-      <c r="G14" s="32">
+      <c r="G14" s="33">
         <f>E14*F14</f>
         <v/>
       </c>
@@ -2887,23 +2988,23 @@
           <t>Engineering-heavy firms</t>
         </is>
       </c>
-      <c r="C15" s="32">
+      <c r="C15" s="33">
         <f>Assumptions!$C$29/Assumptions!$C$85</f>
         <v/>
       </c>
-      <c r="D15" s="33">
+      <c r="D15" s="34">
         <f>Assumptions!$C$33</f>
         <v/>
       </c>
-      <c r="E15" s="32">
+      <c r="E15" s="33">
         <f>C15*D15</f>
         <v/>
       </c>
-      <c r="F15" s="32">
+      <c r="F15" s="33">
         <f>Assumptions!$C$67</f>
         <v/>
       </c>
-      <c r="G15" s="32">
+      <c r="G15" s="33">
         <f>E15*F15</f>
         <v/>
       </c>
@@ -2914,29 +3015,29 @@
           <t>Mid-size structured-hiring firms</t>
         </is>
       </c>
-      <c r="C16" s="32">
+      <c r="C16" s="33">
         <f>Assumptions!$C$30/Assumptions!$C$85</f>
         <v/>
       </c>
-      <c r="D16" s="33">
+      <c r="D16" s="34">
         <f>Assumptions!$C$34</f>
         <v/>
       </c>
-      <c r="E16" s="32">
+      <c r="E16" s="33">
         <f>C16*D16</f>
         <v/>
       </c>
-      <c r="F16" s="32">
+      <c r="F16" s="33">
         <f>Assumptions!$C$68</f>
         <v/>
       </c>
-      <c r="G16" s="32">
+      <c r="G16" s="33">
         <f>E16*F16</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="34" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>TAM  (global prize, full ACV)</t>
         </is>
@@ -2960,22 +3061,22 @@
       <c r="H19" s="5" t="n"/>
     </row>
     <row r="20">
-      <c r="B20" s="18" t="inlineStr">
+      <c r="B20" s="19" t="inlineStr">
         <is>
           <t>CHANNEL ROUTE  (Manatal embedded)</t>
         </is>
       </c>
-      <c r="C20" s="31" t="inlineStr">
+      <c r="C20" s="32" t="inlineStr">
         <is>
           <t>Year 1</t>
         </is>
       </c>
-      <c r="D20" s="31" t="inlineStr">
+      <c r="D20" s="32" t="inlineStr">
         <is>
           <t>Year 2</t>
         </is>
       </c>
-      <c r="E20" s="31" t="inlineStr">
+      <c r="E20" s="32" t="inlineStr">
         <is>
           <t>Year 3</t>
         </is>
@@ -2987,15 +3088,15 @@
           <t>Relevant Manatal clients</t>
         </is>
       </c>
-      <c r="C21" s="32">
+      <c r="C21" s="33">
         <f>(Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72</f>
         <v/>
       </c>
-      <c r="D21" s="32">
+      <c r="D21" s="33">
         <f>(Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72</f>
         <v/>
       </c>
-      <c r="E21" s="32">
+      <c r="E21" s="33">
         <f>(Assumptions!$C$71+Assumptions!$C$76*Assumptions!$C$77)*Assumptions!$C$72</f>
         <v/>
       </c>
@@ -3006,15 +3107,15 @@
           <t>Attach rate</t>
         </is>
       </c>
-      <c r="C22" s="33">
+      <c r="C22" s="34">
         <f>Assumptions!$C$73</f>
         <v/>
       </c>
-      <c r="D22" s="33">
+      <c r="D22" s="34">
         <f>Assumptions!$C$74</f>
         <v/>
       </c>
-      <c r="E22" s="33">
+      <c r="E22" s="34">
         <f>Assumptions!$C$75</f>
         <v/>
       </c>
@@ -3025,21 +3126,21 @@
           <t>Active channel accounts</t>
         </is>
       </c>
-      <c r="C23" s="32">
+      <c r="C23" s="33">
         <f>C21*C22</f>
         <v/>
       </c>
-      <c r="D23" s="32">
+      <c r="D23" s="33">
         <f>D21*D22</f>
         <v/>
       </c>
-      <c r="E23" s="32">
+      <c r="E23" s="33">
         <f>E21*E22</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="B24" s="34" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Channel revenue ($/yr, retention-adj)</t>
         </is>
@@ -3058,14 +3159,14 @@
       </c>
     </row>
     <row r="26">
-      <c r="B26" s="18" t="inlineStr">
+      <c r="B26" s="19" t="inlineStr">
         <is>
           <t>DIRECT ROUTE  (self-serve + sales-led)</t>
         </is>
       </c>
-      <c r="C26" s="19" t="n"/>
-      <c r="D26" s="19" t="n"/>
-      <c r="E26" s="31" t="inlineStr">
+      <c r="C26" s="20" t="n"/>
+      <c r="D26" s="20" t="n"/>
+      <c r="E26" s="32" t="inlineStr">
         <is>
           <t>Year 3</t>
         </is>
@@ -3077,7 +3178,7 @@
           <t>Serviceable SAM accounts</t>
         </is>
       </c>
-      <c r="E27" s="32">
+      <c r="E27" s="33">
         <f>Build!$E$9</f>
         <v/>
       </c>
@@ -3088,7 +3189,7 @@
           <t>3-yr penetration</t>
         </is>
       </c>
-      <c r="E28" s="33">
+      <c r="E28" s="34">
         <f>Assumptions!$C$79</f>
         <v/>
       </c>
@@ -3099,13 +3200,13 @@
           <t>Active direct accounts</t>
         </is>
       </c>
-      <c r="E29" s="32">
+      <c r="E29" s="33">
         <f>E27*E28</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="34" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>Direct revenue ($/yr, retention-adj)</t>
         </is>
@@ -3140,7 +3241,7 @@
     <row r="35" ht="18" customHeight="1">
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>D.  Value delivered  (tests run -&gt; hires -&gt; bad-hire cost addressed)</t>
+          <t>D.  Revenue potential by stream  (assessments + talent-DB)</t>
         </is>
       </c>
       <c r="C35" s="5" t="n"/>
@@ -3151,75 +3252,184 @@
       <c r="H35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="B36" s="31" t="inlineStr">
-        <is>
-          <t>Ring</t>
-        </is>
-      </c>
-      <c r="C36" s="31" t="inlineStr">
-        <is>
-          <t>Accounts</t>
-        </is>
-      </c>
-      <c r="D36" s="31" t="inlineStr">
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Tier</t>
+        </is>
+      </c>
+      <c r="C36" s="32" t="inlineStr">
+        <is>
+          <t>Assessment rev ($/yr)</t>
+        </is>
+      </c>
+      <c r="D36" s="32" t="inlineStr">
         <is>
           <t>Tests run / yr</t>
         </is>
       </c>
-      <c r="E36" s="31" t="inlineStr">
-        <is>
-          <t>Hires supported / yr</t>
-        </is>
-      </c>
-      <c r="F36" s="31" t="inlineStr">
-        <is>
-          <t>Bad-hire $ exposure influenced</t>
-        </is>
-      </c>
-      <c r="G36" s="31" t="inlineStr">
-        <is>
-          <t>Mitigable value to buyers ($)</t>
+      <c r="E36" s="32" t="inlineStr">
+        <is>
+          <t>Talent-DB rev ($/yr)</t>
+        </is>
+      </c>
+      <c r="F36" s="32" t="inlineStr">
+        <is>
+          <t>TOTAL revenue potential ($/yr)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="12" t="inlineStr">
         <is>
+          <t>Full opportunity (TAM)</t>
+        </is>
+      </c>
+      <c r="C37" s="33">
+        <f>Build!$G$17</f>
+        <v/>
+      </c>
+      <c r="D37" s="33">
+        <f>C37/Assumptions!$C$50</f>
+        <v/>
+      </c>
+      <c r="E37" s="33">
+        <f>D37*Assumptions!$C$91*Assumptions!$C$92</f>
+        <v/>
+      </c>
+      <c r="F37" s="36">
+        <f>C37+E37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>Serviceable today (SAM)</t>
+        </is>
+      </c>
+      <c r="C38" s="33">
+        <f>Build!$H$9</f>
+        <v/>
+      </c>
+      <c r="D38" s="33">
+        <f>C38/Assumptions!$C$50</f>
+        <v/>
+      </c>
+      <c r="E38" s="33">
+        <f>D38*Assumptions!$C$91*Assumptions!$C$92</f>
+        <v/>
+      </c>
+      <c r="F38" s="36">
+        <f>C38+E38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>3-yr reachable (SOM)</t>
+        </is>
+      </c>
+      <c r="C39" s="33">
+        <f>Build!$E$33</f>
+        <v/>
+      </c>
+      <c r="D39" s="33">
+        <f>C39/Assumptions!$C$50</f>
+        <v/>
+      </c>
+      <c r="E39" s="33">
+        <f>D39*Assumptions!$C$91*Assumptions!$C$92</f>
+        <v/>
+      </c>
+      <c r="F39" s="36">
+        <f>C39+E39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>E.  Value delivered  (tests run -&gt; hires -&gt; bad-hire cost addressed)</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="n"/>
+      <c r="D41" s="5" t="n"/>
+      <c r="E41" s="5" t="n"/>
+      <c r="F41" s="5" t="n"/>
+      <c r="G41" s="5" t="n"/>
+      <c r="H41" s="5" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="32" t="inlineStr">
+        <is>
+          <t>Ring</t>
+        </is>
+      </c>
+      <c r="C42" s="32" t="inlineStr">
+        <is>
+          <t>Accounts</t>
+        </is>
+      </c>
+      <c r="D42" s="32" t="inlineStr">
+        <is>
+          <t>Tests run / yr</t>
+        </is>
+      </c>
+      <c r="E42" s="32" t="inlineStr">
+        <is>
+          <t>Hires supported / yr</t>
+        </is>
+      </c>
+      <c r="F42" s="32" t="inlineStr">
+        <is>
+          <t>Bad-hire $ exposure influenced</t>
+        </is>
+      </c>
+      <c r="G42" s="32" t="inlineStr">
+        <is>
+          <t>Mitigable value to buyers ($)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="12" t="inlineStr">
+        <is>
           <t>SOM (yr 3)</t>
         </is>
       </c>
-      <c r="C37" s="32">
+      <c r="C43" s="33">
         <f>(Build!$E$23+Build!$E$29)</f>
         <v/>
       </c>
-      <c r="D37" s="32">
-        <f>C37*Assumptions!$C$64</f>
-        <v/>
-      </c>
-      <c r="E37" s="32">
-        <f>D37/Assumptions!$C$88</f>
-        <v/>
-      </c>
-      <c r="F37" s="32">
-        <f>E37*Assumptions!$C$87</f>
-        <v/>
-      </c>
-      <c r="G37" s="32">
-        <f>F37*Assumptions!$C$89</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="B39" s="21" t="inlineStr">
+      <c r="D43" s="33">
+        <f>C43*Assumptions!$C$64</f>
+        <v/>
+      </c>
+      <c r="E43" s="33">
+        <f>D43/Assumptions!$C$88</f>
+        <v/>
+      </c>
+      <c r="F43" s="33">
+        <f>E43*Assumptions!$C$87</f>
+        <v/>
+      </c>
+      <c r="G43" s="33">
+        <f>F43*Assumptions!$C$89</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" s="22" t="inlineStr">
         <is>
           <t>Notes: (1) MECE - agencies and the firms they serve are distinct buyers; agency tests cover client roles, in-house tests cover own roles, no double count. (2) Channel (Manatal, global) and Direct (focus-6) may overlap modestly; treated as additive (slightly optimistic) and flagged. (3) Value-delivered ring is buyer-side: $ exposure influenced and mitigable value are NOT market size - they show the value pool Invirtus serves, against which the SOM revenue captured (~$2.2M) is a tiny slice. (4) Hires = gross placements assessment touches; agencies place for many clients, so per-account hires run high.</t>
         </is>
       </c>
     </row>
-    <row r="40"/>
+    <row r="46"/>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B39:H40"/>
+    <mergeCell ref="B45:H46"/>
     <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3245,14 +3455,14 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>INVIRTUS  -  Sensitivity</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>SOM (Yr3) response to the three swing inputs. Tables recompute the SOM chain live from the axis values; non-swung drivers pull from Assumptions.</t>
         </is>
@@ -3574,22 +3784,22 @@
       </c>
     </row>
     <row r="23">
-      <c r="B23" s="31" t="inlineStr">
+      <c r="B23" s="32" t="inlineStr">
         <is>
           <t>Driver</t>
         </is>
       </c>
-      <c r="C23" s="31" t="inlineStr">
+      <c r="C23" s="32" t="inlineStr">
         <is>
           <t>Low case</t>
         </is>
       </c>
-      <c r="D23" s="31" t="inlineStr">
+      <c r="D23" s="32" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="E23" s="31" t="inlineStr">
+      <c r="E23" s="32" t="inlineStr">
         <is>
           <t>High case</t>
         </is>
@@ -3679,46 +3889,46 @@
   </cols>
   <sheetData>
     <row r="2">
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="17" t="inlineStr">
         <is>
           <t>INVIRTUS  -  Sources</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="17" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>One row per researched input. Figures triangulated where official counts are absent; confidence noted.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="31" t="inlineStr">
+      <c r="B5" s="32" t="inlineStr">
         <is>
           <t>Key</t>
         </is>
       </c>
-      <c r="C5" s="31" t="inlineStr">
+      <c r="C5" s="32" t="inlineStr">
         <is>
           <t>Input</t>
         </is>
       </c>
-      <c r="D5" s="31" t="inlineStr">
+      <c r="D5" s="32" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="32" t="inlineStr">
         <is>
           <t>URL</t>
         </is>
       </c>
-      <c r="F5" s="31" t="inlineStr">
+      <c r="F5" s="32" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="G5" s="31" t="inlineStr">
+      <c r="G5" s="32" t="inlineStr">
         <is>
           <t>Conf.</t>
         </is>
@@ -4013,7 +4223,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="21" t="inlineStr">
+      <c r="B16" s="22" t="inlineStr">
         <is>
           <t>Methodology note: 'medium enterprise' bands differ by country (KSA 50-249 emp; Morocco turnover-based 50-175M MAD; UAE &lt;200 emp; Egypt 50+ emp census band). Mid-size counts are the closest official proxy x an engineer-hiring share. The engineer-hiring share and use-case-fit % are the softest inputs - pressure-test before locking TAM.</t>
         </is>

</xml_diff>

<commit_message>
Make breadth modes a clean ramp; simplify comment tone
- Breadth modes now monotonic: 1 engineers only, 2 some white-collar
  (engineers + adjacent roles), 3 all white-collar. Mode 2 is the
  "more than engineers, less than all" case. Full opportunity:
  $1.11B / $2.41B / $4.98B.
- Trimmed assumption notes, section banners, and cover prose to a plainer,
  shorter tone; removed over-explaining. 0 formula error cells.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RsCNYhV2EbucLSqzkWAFLN
</commit_message>
<xml_diff>
--- a/Invirtus_Market_Sizing.xlsx
+++ b/Invirtus_Market_Sizing.xlsx
@@ -639,7 +639,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:E36"/>
+  <dimension ref="B2:E34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -667,7 +667,7 @@
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Candidate assessment platform  -  decision intelligence layer above the ATS  |  USD  |  Built 2026-06-16</t>
+          <t>Candidate assessment platform  |  USD  |  June 2026</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
     <row r="7">
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Lead with the 3-year reachable number. It runs on two streams - assessment packs plus talent-DB monetization - and is driven first by the Manatal channel (embedded attach ~59% of the assessment line), then self-serve. The single biggest assumption is the Year-3 channel attach rate on the ICP-relevant Manatal base (Assumptions sec. 7); tests/account and the $14 PAYG price are the next two swing factors (see Sensitivity).</t>
+          <t>The 3-year reachable number runs on two streams: assessment packs and talent-DB. The assessment line is channel-led (partner portfolio ~76%, direct ~24%). The biggest swing is the channel attach scalar, then tests/account and price (see Sensitivity).</t>
         </is>
       </c>
       <c r="C7" s="7" t="n"/>
@@ -859,64 +859,48 @@
     <row r="29">
       <c r="B29" s="16" t="inlineStr">
         <is>
-          <t>1.  Every blue cell on Assumptions is an editable input; black cells are formulas with no hardcodes.</t>
+          <t>1.  Blue cells are inputs; black cells are formulas.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" s="16" t="inlineStr">
         <is>
-          <t>2.  Market BREADTH toggle (1 Engineers / 2 White-collar / 3 Narrower) scales the universe; the</t>
+          <t>2.  Breadth toggle (1 engineers / 2 some white-collar / 3 all white-collar) scales the universe.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="B31" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">     headline above reflects the active mode. Channel is a partner PORTFOLIO (Manatal + others), each toggleable.</t>
+          <t>3.  Channel is a partner portfolio (Assumptions sec.7); each partner can be switched on or off.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="B32" s="16" t="inlineStr">
         <is>
-          <t>3.  Build derives Serviceable bottoms-up (entities x %fit x tests/yr x net $/test), grosses up to Full</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     opportunity, and captures the 3-yr figure via the partner channel + direct self-serve/sales, two streams.</t>
+          <t>4.  Two streams: assessment packs + talent-DB. Sources lists the researched inputs.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="B34" s="16" t="inlineStr">
-        <is>
-          <t>4.  Sensitivity flexes the inputs that move it most; Sources lists every researched figure.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="17" t="inlineStr">
+      <c r="B34" s="17" t="inlineStr">
         <is>
           <t>Input (editable)</t>
         </is>
       </c>
-      <c r="C36" s="12" t="inlineStr">
+      <c r="C34" s="12" t="inlineStr">
         <is>
           <t>Formula (calc)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="5">
     <mergeCell ref="B31:E31"/>
     <mergeCell ref="B30:E30"/>
     <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B33:E33"/>
-    <mergeCell ref="B34:E34"/>
     <mergeCell ref="B7:E9"/>
     <mergeCell ref="B32:E32"/>
   </mergeCells>
@@ -987,7 +971,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>1.  Addressable entities  (bottoms-up universe)  [RESEARCH]</t>
+          <t>1.  Addressable entities  (researched)</t>
         </is>
       </c>
       <c r="C5" s="5" t="n"/>
@@ -1027,7 +1011,7 @@
       </c>
       <c r="F7" s="23" t="inlineStr">
         <is>
-          <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
+          <t>Tech/IT recruitment agencies.</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1036,7 @@
       </c>
       <c r="F8" s="23" t="inlineStr">
         <is>
-          <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
+          <t>Tech/IT recruitment agencies.</t>
         </is>
       </c>
     </row>
@@ -1077,7 +1061,7 @@
       </c>
       <c r="F9" s="23" t="inlineStr">
         <is>
-          <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
+          <t>Tech/IT recruitment agencies.</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1086,7 @@
       </c>
       <c r="F10" s="23" t="inlineStr">
         <is>
-          <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
+          <t>Tech/IT recruitment agencies.</t>
         </is>
       </c>
     </row>
@@ -1127,7 +1111,7 @@
       </c>
       <c r="F11" s="23" t="inlineStr">
         <is>
-          <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
+          <t>Tech/IT recruitment agencies.</t>
         </is>
       </c>
     </row>
@@ -1152,7 +1136,7 @@
       </c>
       <c r="F12" s="23" t="inlineStr">
         <is>
-          <t>Recruitment/staffing firms with a tech/IT desk. Tech subset of national agency base.</t>
+          <t>Tech/IT recruitment agencies.</t>
         </is>
       </c>
     </row>
@@ -1188,7 +1172,7 @@
       </c>
       <c r="F14" s="23" t="inlineStr">
         <is>
-          <t>Tech/software/ICT companies that hire engineers in-house.</t>
+          <t>Tech/software/ICT companies.</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1197,7 @@
       </c>
       <c r="F15" s="23" t="inlineStr">
         <is>
-          <t>Tech/software/ICT companies that hire engineers in-house.</t>
+          <t>Tech/software/ICT companies.</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1222,7 @@
       </c>
       <c r="F16" s="23" t="inlineStr">
         <is>
-          <t>Tech/software/ICT companies that hire engineers in-house.</t>
+          <t>Tech/software/ICT companies.</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1247,7 @@
       </c>
       <c r="F17" s="23" t="inlineStr">
         <is>
-          <t>Tech/software/ICT companies that hire engineers in-house.</t>
+          <t>Tech/software/ICT companies.</t>
         </is>
       </c>
     </row>
@@ -1288,7 +1272,7 @@
       </c>
       <c r="F18" s="23" t="inlineStr">
         <is>
-          <t>Tech/software/ICT companies that hire engineers in-house.</t>
+          <t>Tech/software/ICT companies.</t>
         </is>
       </c>
     </row>
@@ -1313,7 +1297,7 @@
       </c>
       <c r="F19" s="23" t="inlineStr">
         <is>
-          <t>Tech/software/ICT companies that hire engineers in-house.</t>
+          <t>Tech/software/ICT companies.</t>
         </is>
       </c>
     </row>
@@ -1349,7 +1333,7 @@
       </c>
       <c r="F21" s="23" t="inlineStr">
         <is>
-          <t>Medium enterprises x share that run structured engineering hiring.</t>
+          <t>Mid-size firms (50-250) hiring engineers.</t>
         </is>
       </c>
     </row>
@@ -1374,7 +1358,7 @@
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>Medium enterprises x share that run structured engineering hiring.</t>
+          <t>Mid-size firms (50-250) hiring engineers.</t>
         </is>
       </c>
     </row>
@@ -1399,7 +1383,7 @@
       </c>
       <c r="F23" s="23" t="inlineStr">
         <is>
-          <t>Medium enterprises x share that run structured engineering hiring.</t>
+          <t>Mid-size firms (50-250) hiring engineers.</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1408,7 @@
       </c>
       <c r="F24" s="23" t="inlineStr">
         <is>
-          <t>Medium enterprises x share that run structured engineering hiring.</t>
+          <t>Mid-size firms (50-250) hiring engineers.</t>
         </is>
       </c>
     </row>
@@ -1449,7 +1433,7 @@
       </c>
       <c r="F25" s="23" t="inlineStr">
         <is>
-          <t>Medium enterprises x share that run structured engineering hiring.</t>
+          <t>Mid-size firms (50-250) hiring engineers.</t>
         </is>
       </c>
     </row>
@@ -1474,7 +1458,7 @@
       </c>
       <c r="F26" s="23" t="inlineStr">
         <is>
-          <t>Medium enterprises x share that run structured engineering hiring.</t>
+          <t>Mid-size firms (50-250) hiring engineers.</t>
         </is>
       </c>
     </row>
@@ -1558,7 +1542,7 @@
     <row r="31" ht="20" customHeight="1">
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>1b. Market breadth toggle  (1=Engineers, 2=White-collar, 3=Narrower)</t>
+          <t>1b. Market breadth toggle</t>
         </is>
       </c>
       <c r="C31" s="5" t="n"/>
@@ -1583,27 +1567,23 @@
       <c r="E32" s="24" t="inlineStr"/>
       <c r="F32" s="23" t="inlineStr">
         <is>
-          <t>1: tech/eng focus (current). 2: all structured white-collar hiring (Aida's broader view). 3: narrower high-conviction core.</t>
+          <t>1 engineers only, 2 engineers + select white-collar, 3 all white-collar hiring.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Active breadth (label)</t>
+          <t xml:space="preserve">   Active breadth</t>
         </is>
       </c>
       <c r="C33" s="27">
-        <f>CHOOSE(Assumptions!$C$32,"1 Engineers only","2 White-collar hiring","3 Narrower use case")</f>
+        <f>CHOOSE(Assumptions!$C$32,"1 Engineers only","2 Some white-collar","3 All white-collar")</f>
         <v/>
       </c>
       <c r="D33" s="23" t="inlineStr"/>
       <c r="E33" s="24" t="inlineStr"/>
-      <c r="F33" s="23" t="inlineStr">
-        <is>
-          <t>Driven by the toggle above.</t>
-        </is>
-      </c>
+      <c r="F33" s="23" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="B34" s="11" t="inlineStr">
@@ -1618,17 +1598,17 @@
       </c>
       <c r="D34" s="24" t="inlineStr">
         <is>
-          <t>2 White-collar</t>
+          <t>2 Some WC</t>
         </is>
       </c>
       <c r="E34" s="24" t="inlineStr">
         <is>
-          <t>3 Narrower</t>
+          <t>3 All WC</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>Logic</t>
+          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -1642,14 +1622,14 @@
         <v>1</v>
       </c>
       <c r="D35" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E35" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="E35" s="28" t="n">
-        <v>1</v>
-      </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>Tech agencies -&gt; all recruitment agencies (tech ~10-15% of total).</t>
+          <t>Tech agencies are ~10-15% of all recruitment agencies.</t>
         </is>
       </c>
     </row>
@@ -1663,14 +1643,14 @@
         <v>1</v>
       </c>
       <c r="D36" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="28" t="n">
         <v>4</v>
       </c>
-      <c r="E36" s="28" t="n">
-        <v>0.5</v>
-      </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>Tech firms -&gt; all firms with structured white-collar hiring.</t>
+          <t>Tech firms to all firms with structured hiring.</t>
         </is>
       </c>
     </row>
@@ -1684,14 +1664,14 @@
         <v>1</v>
       </c>
       <c r="D37" s="28" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="E37" s="28" t="n">
         <v>3</v>
       </c>
-      <c r="E37" s="28" t="n">
-        <v>0.2</v>
-      </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>Eng-hiring mid-size -&gt; all mid-size structured hirers (2) / core only (3).</t>
+          <t>Engineer-hiring to all mid-size hirers.</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1780,7 @@
       <c r="E43" s="24" t="inlineStr"/>
       <c r="F43" s="23" t="inlineStr">
         <is>
-          <t>Tech recruiting agencies run high req volume; structured assessment is core to their value-add. High fit.</t>
+          <t>Assessment is core to agency workflow.</t>
         </is>
       </c>
     </row>
@@ -1821,7 +1801,7 @@
       <c r="E44" s="24" t="inlineStr"/>
       <c r="F44" s="23" t="inlineStr">
         <is>
-          <t>Broad tech-firm base is ~95% micro (&lt;50 staff, solo dev shops). Only volume hirers run structured multi-candidate evaluation. Deliberately low.</t>
+          <t>Base skews micro; only volume hirers fit.</t>
         </is>
       </c>
     </row>
@@ -1842,14 +1822,14 @@
       <c r="E45" s="24" t="inlineStr"/>
       <c r="F45" s="23" t="inlineStr">
         <is>
-          <t>ICP pain (inconsistent evaluation) but lower adoption propensity / hire sporadically. Conservative.</t>
+          <t>Lower adoption; hire sporadically.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>3.  Pricing  (usage-based: $/test, packs)  [given]</t>
+          <t>3.  Pricing  (usage-based, per test)</t>
         </is>
       </c>
       <c r="C46" s="5" t="n"/>
@@ -1878,7 +1858,7 @@
       </c>
       <c r="F47" s="23" t="inlineStr">
         <is>
-          <t>Finalized BP base (was $15). Benchmark: TestGorilla ~$4.3/candidate, TestDome $7-20, HackerRank $15-20, Adaface entry $15. $14 sits at premium end.</t>
+          <t>From BP. Premium vs TestGorilla (~$4/candidate); near TestDome/HackerRank.</t>
         </is>
       </c>
     </row>
@@ -1897,11 +1877,7 @@
         </is>
       </c>
       <c r="E48" s="24" t="inlineStr"/>
-      <c r="F48" s="23" t="inlineStr">
-        <is>
-          <t>Given.</t>
-        </is>
-      </c>
+      <c r="F48" s="23" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="B49" s="16" t="inlineStr">
@@ -1918,11 +1894,7 @@
         </is>
       </c>
       <c r="E49" s="24" t="inlineStr"/>
-      <c r="F49" s="23" t="inlineStr">
-        <is>
-          <t>Given.</t>
-        </is>
-      </c>
+      <c r="F49" s="23" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="B50" s="16" t="inlineStr">
@@ -1941,7 +1913,7 @@
       <c r="E50" s="24" t="inlineStr"/>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>Finalized BP top tier: 1,000-test Enterprise pack at $11,200 (= $11.20/test). Replaces old 200-unit Large and the flat enterprise fee.</t>
+          <t>1,000-test pack, $11,200 ($11.20/test).</t>
         </is>
       </c>
     </row>
@@ -2020,7 +1992,7 @@
     <row r="55" ht="20" customHeight="1">
       <c r="B55" s="4" t="inlineStr">
         <is>
-          <t>4.  Pack mix  (share of accounts on each plan)  [pack-led per finalized BP]</t>
+          <t>4.  Pack mix</t>
         </is>
       </c>
       <c r="C55" s="5" t="n"/>
@@ -2045,7 +2017,7 @@
       <c r="E56" s="24" t="inlineStr"/>
       <c r="F56" s="23" t="inlineStr">
         <is>
-          <t>Finalized BP is pack-led; PAYG is a thin trial tier, not the base.</t>
+          <t>Pack-led mix; PAYG is a thin trial tier.</t>
         </is>
       </c>
     </row>
@@ -2098,11 +2070,7 @@
         </is>
       </c>
       <c r="E59" s="24" t="inlineStr"/>
-      <c r="F59" s="23" t="inlineStr">
-        <is>
-          <t>Heaviest buyers; matches finalized BP customer mix.</t>
-        </is>
-      </c>
+      <c r="F59" s="23" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="B60" s="16" t="inlineStr">
@@ -2176,7 +2144,7 @@
       <c r="E63" s="24" t="inlineStr"/>
       <c r="F63" s="23" t="inlineStr">
         <is>
-          <t>Global multiplier on tests/account. Base=1.00; flex in sensitivity.</t>
+          <t>Multiplier on tests/account.</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2165,7 @@
       <c r="E64" s="24" t="inlineStr"/>
       <c r="F64" s="23" t="inlineStr">
         <is>
-          <t>High req throughput - many client roles, several candidates screened each.</t>
+          <t>High volume across client roles.</t>
         </is>
       </c>
     </row>
@@ -2236,7 +2204,7 @@
       <c r="E66" s="24" t="inlineStr"/>
       <c r="F66" s="23" t="inlineStr">
         <is>
-          <t>roles x candidates x scalar.</t>
+          <t>Roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
@@ -2257,7 +2225,7 @@
       <c r="E67" s="24" t="inlineStr"/>
       <c r="F67" s="23" t="inlineStr">
         <is>
-          <t>Steady in-house eng hiring.</t>
+          <t>Steady in-house hiring.</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2264,7 @@
       <c r="E69" s="24" t="inlineStr"/>
       <c r="F69" s="23" t="inlineStr">
         <is>
-          <t>roles x candidates x scalar.</t>
+          <t>Roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
@@ -2317,7 +2285,7 @@
       <c r="E70" s="24" t="inlineStr"/>
       <c r="F70" s="23" t="inlineStr">
         <is>
-          <t>Sporadic, lower-volume hiring.</t>
+          <t>Lower-volume hiring.</t>
         </is>
       </c>
     </row>
@@ -2356,7 +2324,7 @@
       <c r="E72" s="24" t="inlineStr"/>
       <c r="F72" s="23" t="inlineStr">
         <is>
-          <t>roles x candidates x scalar.</t>
+          <t>Roles x candidates x scalar.</t>
         </is>
       </c>
     </row>
@@ -2377,7 +2345,7 @@
       <c r="E73" s="24" t="inlineStr"/>
       <c r="F73" s="23" t="inlineStr">
         <is>
-          <t>Manatal users: mix of agencies + in-house recruiters.</t>
+          <t>Mix of agencies and in-house recruiters.</t>
         </is>
       </c>
     </row>
@@ -2518,7 +2486,7 @@
     <row r="81" ht="20" customHeight="1">
       <c r="B81" s="4" t="inlineStr">
         <is>
-          <t>7.  SOM - Channel: partner distribution portfolio  [beyond Manatal]</t>
+          <t>7.  Channel: partner distribution portfolio</t>
         </is>
       </c>
       <c r="C81" s="5" t="n"/>
@@ -2738,7 +2706,7 @@
       <c r="E90" s="24" t="inlineStr"/>
       <c r="F90" s="23" t="inlineStr">
         <is>
-          <t>Global multiplier on all partner attach rates. Base=1.00; flex in sensitivity. (Channel tests/acct &amp; ACV in secs 5-6.)</t>
+          <t>Multiplier on all partner attach rates.</t>
         </is>
       </c>
     </row>
@@ -2770,7 +2738,7 @@
       <c r="E92" s="24" t="inlineStr"/>
       <c r="F92" s="23" t="inlineStr">
         <is>
-          <t>Direct capture is gated by low trial-to-paid; a pre-seed wins only a thin slice of the large serviceable base.</t>
+          <t>Thin slice; gated by low trial-to-paid.</t>
         </is>
       </c>
     </row>
@@ -2791,7 +2759,7 @@
       <c r="E93" s="24" t="inlineStr"/>
       <c r="F93" s="23" t="inlineStr">
         <is>
-          <t>Self-serve funnel cross-check input (year-3 run-rate).</t>
+          <t>Funnel cross-check (year-3 run-rate).</t>
         </is>
       </c>
     </row>
@@ -2833,7 +2801,7 @@
       </c>
       <c r="F95" s="23" t="inlineStr">
         <is>
-          <t>Currently LOW - do NOT assume best-in-class. Flagged in GTM notes.</t>
+          <t>Low today; not best-in-class.</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2837,7 @@
       </c>
       <c r="F97" s="23" t="inlineStr">
         <is>
-          <t>Finalized BP assumes 7% gross churn (93% retention); held slightly conservative at 90% for the SOM. 100% to date on a tiny base.</t>
+          <t>BP uses 7% churn; 90% here. 100% to date on a tiny base.</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2858,7 @@
       <c r="E98" s="24" t="inlineStr"/>
       <c r="F98" s="23" t="inlineStr">
         <is>
-          <t>Focus-6 as % of all geos where product works. Grosses SAM up to TAM. US/India/rest-EU dominate.</t>
+          <t>Focus-6 as % of global; grosses up to full opportunity.</t>
         </is>
       </c>
     </row>
@@ -2926,7 +2894,7 @@
       </c>
       <c r="F100" s="23" t="inlineStr">
         <is>
-          <t>Core value anchor used across sales &amp; fundraising.</t>
+          <t>Value anchor.</t>
         </is>
       </c>
     </row>
@@ -2947,7 +2915,7 @@
       <c r="E101" s="24" t="inlineStr"/>
       <c r="F101" s="23" t="inlineStr">
         <is>
-          <t>Candidates assessed per filled role (1 hire/role).</t>
+          <t>Candidates per hire.</t>
         </is>
       </c>
     </row>
@@ -2968,14 +2936,14 @@
       <c r="E102" s="24" t="inlineStr"/>
       <c r="F102" s="23" t="inlineStr">
         <is>
-          <t>Assumed share of bad-hire cost avoided via better screening.</t>
+          <t>Share of bad-hire cost avoided.</t>
         </is>
       </c>
     </row>
     <row r="103" ht="20" customHeight="1">
       <c r="B103" s="4" t="inlineStr">
         <is>
-          <t>11. Talent-DB monetization  (2nd revenue stream)  [finalized BP]</t>
+          <t>11. Talent-DB monetization  (2nd stream)</t>
         </is>
       </c>
       <c r="C103" s="5" t="n"/>
@@ -3004,7 +2972,7 @@
       </c>
       <c r="F104" s="23" t="inlineStr">
         <is>
-          <t>Finalized BP ramps 1% (2026) -&gt; 50% (2030); 30% used as mature steady-state. Profiles sourced = tests run x this %.</t>
+          <t>BP ramps 1% to 50%; 30% mature. Profiles = tests x this %.</t>
         </is>
       </c>
     </row>
@@ -3029,7 +2997,7 @@
       </c>
       <c r="F105" s="23" t="inlineStr">
         <is>
-          <t>Finalized BP: $30 per sourced profile, flat.</t>
+          <t>$30 per profile (BP).</t>
         </is>
       </c>
     </row>
@@ -3707,7 +3675,7 @@
     <row r="45">
       <c r="B45" s="23" t="inlineStr">
         <is>
-          <t>Notes: (1) MECE - agencies and the firms they serve are distinct buyers; agency tests cover client roles, in-house tests cover own roles, no double count. (2) Channel (Manatal, global) and Direct (focus-6) may overlap modestly; treated as additive (slightly optimistic) and flagged. (3) Value-delivered ring is buyer-side: $ exposure influenced and mitigable value are NOT market size - they show the value pool Invirtus serves, against which the SOM revenue captured (~$2.2M) is a tiny slice. (4) Hires = gross placements assessment touches; agencies place for many clients, so per-account hires run high.</t>
+          <t>Notes: Agencies and the firms they serve are counted separately, so there is no double count. Channel and direct may overlap a little; treated as additive. The value-delivered figures are buyer-side, not market size.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove all TAM/SAM/SOM labels; use revenue-potential language throughout
Renamed the tiers everywhere in the workbook and README to Full opportunity /
Serviceable today / 3-year reachable (no TAM/SAM/SOM tags). Updated section
banners, table titles, tornado, cover cards, and notes accordingly. Internal
Python variable names are unchanged (not user-facing). 0 formula error cells.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RsCNYhV2EbucLSqzkWAFLN
</commit_message>
<xml_diff>
--- a/Invirtus_Market_Sizing.xlsx
+++ b/Invirtus_Market_Sizing.xlsx
@@ -660,7 +660,7 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Bottoms-Up Revenue Potential  (two streams; TAM / SAM / SOM equivalents)</t>
+          <t>Bottoms-Up Revenue Potential  (two streams)</t>
         </is>
       </c>
     </row>
@@ -737,17 +737,17 @@
     <row r="13">
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>(TAM) all geos | 2 streams</t>
+          <t>All geos | 2 streams</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>(SAM) focus-6 | serviceable</t>
+          <t>Focus-6 | serviceable</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>(SOM) channel+direct | 3-yr</t>
+          <t>Channel + direct | 3-yr</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
     <row r="91" ht="20" customHeight="1">
       <c r="B91" s="4" t="inlineStr">
         <is>
-          <t>8.  SOM - Direct route (self-serve + sales-led)</t>
+          <t>8.  Direct route (self-serve + sales-led)</t>
         </is>
       </c>
       <c r="C91" s="5" t="n"/>
@@ -2724,7 +2724,7 @@
     <row r="92">
       <c r="B92" s="16" t="inlineStr">
         <is>
-          <t>3-yr penetration of serviceable SAM accounts</t>
+          <t>3-yr penetration of serviceable accounts</t>
         </is>
       </c>
       <c r="C92" s="29" t="n">
@@ -3031,7 +3031,7 @@
     <row r="1">
       <c r="B1" s="18" t="inlineStr">
         <is>
-          <t>INVIRTUS  -  Revenue potential build  (TAM / SAM / SOM)</t>
+          <t>INVIRTUS  -  Revenue potential build</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3045,7 @@
     <row r="4" ht="18" customHeight="1">
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>A.  Serviceable accounts  (focus-6 = SAM geography)</t>
+          <t>A.  Serviceable accounts  (focus-6 geos)</t>
         </is>
       </c>
       <c r="C4" s="5" t="n"/>
@@ -3088,7 +3088,7 @@
       </c>
       <c r="H5" s="38" t="inlineStr">
         <is>
-          <t>SAM value ($/yr)</t>
+          <t>Value ($/yr)</t>
         </is>
       </c>
     </row>
@@ -3188,7 +3188,7 @@
     <row r="9">
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>SAM  (focus-6, serviceable today)</t>
+          <t>Serviceable today  (focus-6)</t>
         </is>
       </c>
       <c r="E9" s="37">
@@ -3203,7 +3203,7 @@
     <row r="11" ht="18" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>B.  TAM  (all geos where product works, at full ACV)</t>
+          <t>B.  Full opportunity  (all geos where product works, full ACV)</t>
         </is>
       </c>
       <c r="C11" s="5" t="n"/>
@@ -3248,7 +3248,7 @@
       </c>
       <c r="G13" s="38" t="inlineStr">
         <is>
-          <t>TAM value ($/yr)</t>
+          <t>Value ($/yr)</t>
         </is>
       </c>
     </row>
@@ -3336,7 +3336,7 @@
     <row r="17">
       <c r="B17" s="14" t="inlineStr">
         <is>
-          <t>TAM  (global prize, full ACV)</t>
+          <t>Full opportunity  (all geos, full ACV)</t>
         </is>
       </c>
       <c r="G17" s="37">
@@ -3347,7 +3347,7 @@
     <row r="19" ht="18" customHeight="1">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>C.  SOM  (3-year reachable)  -  two routes side by side</t>
+          <t>C.  3-year reachable  -  two routes side by side</t>
         </is>
       </c>
       <c r="C19" s="5" t="n"/>
@@ -3428,7 +3428,7 @@
     <row r="27">
       <c r="B27" s="12" t="inlineStr">
         <is>
-          <t>Serviceable SAM accounts</t>
+          <t>Serviceable accounts</t>
         </is>
       </c>
       <c r="E27" s="36">
@@ -3483,7 +3483,7 @@
     <row r="33">
       <c r="B33" s="43" t="inlineStr">
         <is>
-          <t>SOM  (Year 3 = Channel + Direct)</t>
+          <t>3-year reachable  (Channel + Direct)</t>
         </is>
       </c>
       <c r="E33" s="44">
@@ -3534,7 +3534,7 @@
     <row r="37">
       <c r="B37" s="12" t="inlineStr">
         <is>
-          <t>Full opportunity (TAM)</t>
+          <t>Full opportunity</t>
         </is>
       </c>
       <c r="C37" s="36">
@@ -3557,7 +3557,7 @@
     <row r="38">
       <c r="B38" s="12" t="inlineStr">
         <is>
-          <t>Serviceable today (SAM)</t>
+          <t>Serviceable today</t>
         </is>
       </c>
       <c r="C38" s="36">
@@ -3580,7 +3580,7 @@
     <row r="39">
       <c r="B39" s="12" t="inlineStr">
         <is>
-          <t>3-yr reachable (SOM)</t>
+          <t>3-yr reachable</t>
         </is>
       </c>
       <c r="C39" s="36">
@@ -3648,7 +3648,7 @@
     <row r="43">
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t>SOM (yr 3)</t>
+          <t>3-yr reachable</t>
         </is>
       </c>
       <c r="C43" s="36">
@@ -3717,14 +3717,14 @@
     <row r="3">
       <c r="B3" s="19" t="inlineStr">
         <is>
-          <t>SOM (Yr3) response to the three swing inputs. Tables recompute the SOM chain live from the axis values; non-swung drivers pull from Assumptions.</t>
+          <t>3-yr reachable revenue response to the three swing inputs. Tables recompute it live from the axis values; other drivers pull from Assumptions.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Table 1:  SOM (Yr3)  -  Channel tests/account  vs  PAYG price/test</t>
+          <t>Table 1:  Channel tests/account  vs  PAYG price/test</t>
         </is>
       </c>
     </row>
@@ -3878,7 +3878,7 @@
     <row r="13">
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Table 2:  SOM (Yr3)  -  Channel attach scalar  vs  Channel tests/account</t>
+          <t>Table 2:  Channel attach scalar  vs  Channel tests/account</t>
         </is>
       </c>
     </row>
@@ -4032,7 +4032,7 @@
     <row r="22">
       <c r="B22" s="11" t="inlineStr">
         <is>
-          <t>Tornado:  SOM swing from +/- moves in each driver</t>
+          <t>Tornado:  swing from +/- moves in each driver</t>
         </is>
       </c>
     </row>
@@ -4478,7 +4478,7 @@
     <row r="16">
       <c r="B16" s="23" t="inlineStr">
         <is>
-          <t>Methodology note: 'medium enterprise' bands differ by country (KSA 50-249 emp; Morocco turnover-based 50-175M MAD; UAE &lt;200 emp; Egypt 50+ emp census band). Mid-size counts are the closest official proxy x an engineer-hiring share. The engineer-hiring share and use-case-fit % are the softest inputs - pressure-test before locking TAM.</t>
+          <t>Methodology note: 'medium enterprise' bands differ by country (KSA 50-249 emp; Morocco turnover-based 50-175M MAD; UAE &lt;200 emp; Egypt 50+ emp census band). Mid-size counts are the closest official proxy x an engineer-hiring share. The engineer-hiring share and use-case-fit % are the softest inputs - pressure-test before widening breadth.</t>
         </is>
       </c>
     </row>

</xml_diff>